<commit_message>
feat: real dataset sample + flexible column analysis (any format)
</commit_message>
<xml_diff>
--- a/backend/data/sample-campaign-skincare.xlsx
+++ b/backend/data/sample-campaign-skincare.xlsx
@@ -3,7 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Campaign Data" sheetId="1" r:id="rId1"/>
+    <sheet name="Chiến dịch Marketing" sheetId="1" r:id="rId1"/>
+    <sheet name="Thông tin nguồn" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -397,46 +398,54 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I91"/>
+  <dimension ref="A1:K91"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="10.83203125" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="24.83203125" customWidth="1"/>
+    <col min="5" max="5" width="26.83203125" customWidth="1"/>
+    <col min="6" max="6" width="22.83203125" customWidth="1"/>
+    <col min="7" max="7" width="10.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="16.83203125" customWidth="1"/>
+    <col min="10" max="10" width="22.83203125" customWidth="1"/>
+    <col min="11" max="11" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Date</v>
+        <v>Ngày</v>
       </c>
       <c r="B1" t="str">
-        <v>Revenue</v>
+        <v>Doanh thu (VND)</v>
       </c>
       <c r="C1" t="str">
-        <v>UnitsSold</v>
+        <v>Số đơn bán</v>
       </c>
       <c r="D1" t="str">
-        <v>PostsPublished</v>
+        <v>Chi phí QC YouTube (VND)</v>
       </c>
       <c r="E1" t="str">
-        <v>AIContentPct</v>
+        <v>Chi phí QC Facebook (VND)</v>
       </c>
       <c r="F1" t="str">
-        <v>Reach</v>
+        <v>Tổng chi phí QC (VND)</v>
       </c>
       <c r="G1" t="str">
-        <v>EngagementRate</v>
+        <v>ROI (%)</v>
       </c>
       <c r="H1" t="str">
-        <v>Clicks</v>
+        <v>Số bài đăng</v>
       </c>
       <c r="I1" t="str">
-        <v>Platform</v>
+        <v>Lượt tiếp cận</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Tỷ lệ tương tác (%)</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Lượt click</v>
       </c>
     </row>
     <row r="2">
@@ -444,28 +453,34 @@
         <v>2026-02-01</v>
       </c>
       <c r="B2">
-        <v>5152880</v>
+        <v>26751969</v>
       </c>
       <c r="C2">
-        <v>50</v>
+        <v>223</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>2789619</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>2748249</v>
       </c>
       <c r="F2">
-        <v>229</v>
+        <v>5537868</v>
       </c>
       <c r="G2">
-        <v>1.37</v>
+        <v>383.1</v>
       </c>
       <c r="H2">
-        <v>12</v>
-      </c>
-      <c r="I2" t="str">
-        <v/>
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>12145</v>
+      </c>
+      <c r="J2">
+        <v>6.31</v>
+      </c>
+      <c r="K2">
+        <v>766</v>
       </c>
     </row>
     <row r="3">
@@ -473,28 +488,34 @@
         <v>2026-02-02</v>
       </c>
       <c r="B3">
-        <v>6570461</v>
+        <v>15236220</v>
       </c>
       <c r="C3">
-        <v>69</v>
+        <v>127</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>389631</v>
       </c>
       <c r="E3">
-        <v>41</v>
+        <v>2062561</v>
       </c>
       <c r="F3">
-        <v>6993</v>
+        <v>2452192</v>
       </c>
       <c r="G3">
-        <v>5.51</v>
+        <v>521.3</v>
       </c>
       <c r="H3">
-        <v>2312</v>
-      </c>
-      <c r="I3" t="str">
-        <v>facebook</v>
+        <v>2</v>
+      </c>
+      <c r="I3">
+        <v>12508</v>
+      </c>
+      <c r="J3">
+        <v>6.46</v>
+      </c>
+      <c r="K3">
+        <v>808</v>
       </c>
     </row>
     <row r="4">
@@ -502,28 +523,34 @@
         <v>2026-02-03</v>
       </c>
       <c r="B4">
-        <v>4532389</v>
+        <v>14153543</v>
       </c>
       <c r="C4">
-        <v>43</v>
+        <v>118</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>130644</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>2086001</v>
       </c>
       <c r="F4">
-        <v>326</v>
+        <v>2216645</v>
       </c>
       <c r="G4">
-        <v>1.86</v>
+        <v>538.5</v>
       </c>
       <c r="H4">
-        <v>5</v>
-      </c>
-      <c r="I4" t="str">
-        <v>instagram</v>
+        <v>2</v>
+      </c>
+      <c r="I4">
+        <v>14105</v>
+      </c>
+      <c r="J4">
+        <v>7.13</v>
+      </c>
+      <c r="K4">
+        <v>1006</v>
       </c>
     </row>
     <row r="5">
@@ -531,28 +558,34 @@
         <v>2026-02-04</v>
       </c>
       <c r="B5">
-        <v>5352638</v>
+        <v>23208661</v>
       </c>
       <c r="C5">
-        <v>56</v>
+        <v>193</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>1699722</v>
       </c>
       <c r="E5">
-        <v>42</v>
+        <v>2775712</v>
       </c>
       <c r="F5">
-        <v>5054</v>
+        <v>4475434</v>
       </c>
       <c r="G5">
-        <v>3.42</v>
+        <v>418.6</v>
       </c>
       <c r="H5">
-        <v>519</v>
-      </c>
-      <c r="I5" t="str">
-        <v>both</v>
+        <v>2</v>
+      </c>
+      <c r="I5">
+        <v>12992</v>
+      </c>
+      <c r="J5">
+        <v>6.66</v>
+      </c>
+      <c r="K5">
+        <v>865</v>
       </c>
     </row>
     <row r="6">
@@ -560,28 +593,34 @@
         <v>2026-02-05</v>
       </c>
       <c r="B6">
-        <v>4502803</v>
+        <v>17696850</v>
       </c>
       <c r="C6">
-        <v>46</v>
+        <v>147</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>2206407</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>815992</v>
       </c>
       <c r="F6">
-        <v>229</v>
+        <v>3022399</v>
       </c>
       <c r="G6">
-        <v>1.46</v>
+        <v>485.5</v>
       </c>
       <c r="H6">
-        <v>13</v>
-      </c>
-      <c r="I6" t="str">
-        <v>facebook</v>
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>5613</v>
+      </c>
+      <c r="J6">
+        <v>3.59</v>
+      </c>
+      <c r="K6">
+        <v>202</v>
       </c>
     </row>
     <row r="7">
@@ -589,28 +628,34 @@
         <v>2026-02-06</v>
       </c>
       <c r="B7">
-        <v>6339014</v>
+        <v>12086614</v>
       </c>
       <c r="C7">
-        <v>61</v>
+        <v>101</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>51809</v>
       </c>
       <c r="E7">
-        <v>43</v>
+        <v>1741197</v>
       </c>
       <c r="F7">
-        <v>4855</v>
+        <v>1793006</v>
       </c>
       <c r="G7">
-        <v>4.29</v>
+        <v>574.1</v>
       </c>
       <c r="H7">
-        <v>833</v>
-      </c>
-      <c r="I7" t="str">
-        <v>instagram</v>
+        <v>2</v>
+      </c>
+      <c r="I7">
+        <v>14831</v>
+      </c>
+      <c r="J7">
+        <v>7.43</v>
+      </c>
+      <c r="K7">
+        <v>1102</v>
       </c>
     </row>
     <row r="8">
@@ -618,28 +663,34 @@
         <v>2026-02-07</v>
       </c>
       <c r="B8">
-        <v>5071737</v>
+        <v>16614173</v>
       </c>
       <c r="C8">
-        <v>48</v>
+        <v>138</v>
       </c>
       <c r="D8">
-        <v>0</v>
+        <v>624604</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>2140936</v>
       </c>
       <c r="F8">
-        <v>349</v>
+        <v>2765540</v>
       </c>
       <c r="G8">
-        <v>0.84</v>
+        <v>500.8</v>
       </c>
       <c r="H8">
-        <v>8</v>
-      </c>
-      <c r="I8" t="str">
-        <v/>
+        <v>2</v>
+      </c>
+      <c r="I8">
+        <v>10935</v>
+      </c>
+      <c r="J8">
+        <v>5.81</v>
+      </c>
+      <c r="K8">
+        <v>635</v>
       </c>
     </row>
     <row r="9">
@@ -647,28 +698,34 @@
         <v>2026-02-08</v>
       </c>
       <c r="B9">
-        <v>4357390</v>
+        <v>17992126</v>
       </c>
       <c r="C9">
-        <v>39</v>
+        <v>150</v>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>1555091</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>1538988</v>
       </c>
       <c r="F9">
-        <v>149</v>
+        <v>3094079</v>
       </c>
       <c r="G9">
-        <v>1.59</v>
+        <v>481.5</v>
       </c>
       <c r="H9">
-        <v>19</v>
-      </c>
-      <c r="I9" t="str">
-        <v/>
+        <v>2</v>
+      </c>
+      <c r="I9">
+        <v>7742</v>
+      </c>
+      <c r="J9">
+        <v>4.48</v>
+      </c>
+      <c r="K9">
+        <v>347</v>
       </c>
     </row>
     <row r="10">
@@ -676,28 +733,34 @@
         <v>2026-02-09</v>
       </c>
       <c r="B10">
-        <v>6013815</v>
+        <v>9724409</v>
       </c>
       <c r="C10">
-        <v>53</v>
+        <v>81</v>
       </c>
       <c r="D10">
-        <v>1</v>
+        <v>484673</v>
       </c>
       <c r="E10">
-        <v>44</v>
+        <v>866024</v>
       </c>
       <c r="F10">
-        <v>5849</v>
+        <v>1350697</v>
       </c>
       <c r="G10">
-        <v>7.33</v>
+        <v>620</v>
       </c>
       <c r="H10">
-        <v>1715</v>
-      </c>
-      <c r="I10" t="str">
-        <v>facebook</v>
+        <v>2</v>
+      </c>
+      <c r="I10">
+        <v>3508</v>
+      </c>
+      <c r="J10">
+        <v>2.71</v>
+      </c>
+      <c r="K10">
+        <v>95</v>
       </c>
     </row>
     <row r="11">
@@ -705,28 +768,34 @@
         <v>2026-02-10</v>
       </c>
       <c r="B11">
-        <v>4845980</v>
+        <v>15433071</v>
       </c>
       <c r="C11">
-        <v>43</v>
+        <v>129</v>
       </c>
       <c r="D11">
+        <v>2286317</v>
+      </c>
+      <c r="E11">
+        <v>209709</v>
+      </c>
+      <c r="F11">
+        <v>2496026</v>
+      </c>
+      <c r="G11">
+        <v>518.3</v>
+      </c>
+      <c r="H11">
         <v>0</v>
       </c>
-      <c r="E11">
-        <v>0</v>
-      </c>
-      <c r="F11">
-        <v>225</v>
-      </c>
-      <c r="G11">
-        <v>1.3</v>
-      </c>
-      <c r="H11">
-        <v>7</v>
-      </c>
-      <c r="I11" t="str">
-        <v>instagram</v>
+      <c r="I11">
+        <v>3629</v>
+      </c>
+      <c r="J11">
+        <v>2.76</v>
+      </c>
+      <c r="K11">
+        <v>100</v>
       </c>
     </row>
     <row r="12">
@@ -734,28 +803,34 @@
         <v>2026-02-11</v>
       </c>
       <c r="B12">
-        <v>6294613</v>
+        <v>13464567</v>
       </c>
       <c r="C12">
-        <v>63</v>
+        <v>112</v>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>1324730</v>
       </c>
       <c r="E12">
-        <v>45</v>
+        <v>746905</v>
       </c>
       <c r="F12">
-        <v>6982</v>
+        <v>2071635</v>
       </c>
       <c r="G12">
-        <v>6.31</v>
+        <v>549.9</v>
       </c>
       <c r="H12">
-        <v>2643</v>
-      </c>
-      <c r="I12" t="str">
-        <v>both</v>
+        <v>2</v>
+      </c>
+      <c r="I12">
+        <v>4403</v>
+      </c>
+      <c r="J12">
+        <v>3.08</v>
+      </c>
+      <c r="K12">
+        <v>136</v>
       </c>
     </row>
     <row r="13">
@@ -763,28 +838,34 @@
         <v>2026-02-12</v>
       </c>
       <c r="B13">
-        <v>4307164</v>
+        <v>22125984</v>
       </c>
       <c r="C13">
-        <v>43</v>
+        <v>184</v>
       </c>
       <c r="D13">
-        <v>0</v>
+        <v>2489511</v>
       </c>
       <c r="E13">
-        <v>0</v>
+        <v>1681324</v>
       </c>
       <c r="F13">
-        <v>294</v>
+        <v>4170835</v>
       </c>
       <c r="G13">
-        <v>0.73</v>
+        <v>430.5</v>
       </c>
       <c r="H13">
-        <v>13</v>
-      </c>
-      <c r="I13" t="str">
-        <v>facebook</v>
+        <v>2</v>
+      </c>
+      <c r="I13">
+        <v>8806</v>
+      </c>
+      <c r="J13">
+        <v>4.92</v>
+      </c>
+      <c r="K13">
+        <v>433</v>
       </c>
     </row>
     <row r="14">
@@ -792,28 +873,34 @@
         <v>2026-02-13</v>
       </c>
       <c r="B14">
-        <v>6182450</v>
+        <v>14055118</v>
       </c>
       <c r="C14">
-        <v>62</v>
+        <v>117</v>
       </c>
       <c r="D14">
-        <v>1</v>
+        <v>222842</v>
       </c>
       <c r="E14">
-        <v>46</v>
+        <v>1972855</v>
       </c>
       <c r="F14">
-        <v>4207</v>
+        <v>2195697</v>
       </c>
       <c r="G14">
-        <v>7.03</v>
+        <v>540.1</v>
       </c>
       <c r="H14">
-        <v>1775</v>
-      </c>
-      <c r="I14" t="str">
-        <v>instagram</v>
+        <v>2</v>
+      </c>
+      <c r="I14">
+        <v>11492</v>
+      </c>
+      <c r="J14">
+        <v>6.04</v>
+      </c>
+      <c r="K14">
+        <v>694</v>
       </c>
     </row>
     <row r="15">
@@ -821,28 +908,34 @@
         <v>2026-02-14</v>
       </c>
       <c r="B15">
-        <v>5124856</v>
+        <v>14547244</v>
       </c>
       <c r="C15">
-        <v>50</v>
+        <v>121</v>
       </c>
       <c r="D15">
-        <v>0</v>
+        <v>1542866</v>
       </c>
       <c r="E15">
-        <v>0</v>
+        <v>758348</v>
       </c>
       <c r="F15">
-        <v>122</v>
+        <v>2301214</v>
       </c>
       <c r="G15">
-        <v>1.4</v>
+        <v>532.2</v>
       </c>
       <c r="H15">
-        <v>4</v>
-      </c>
-      <c r="I15" t="str">
-        <v/>
+        <v>2</v>
+      </c>
+      <c r="I15">
+        <v>4839</v>
+      </c>
+      <c r="J15">
+        <v>3.27</v>
+      </c>
+      <c r="K15">
+        <v>158</v>
       </c>
     </row>
     <row r="16">
@@ -850,28 +943,34 @@
         <v>2026-02-15</v>
       </c>
       <c r="B16">
-        <v>4731513</v>
+        <v>23700787</v>
       </c>
       <c r="C16">
-        <v>41</v>
+        <v>198</v>
       </c>
       <c r="D16">
-        <v>0</v>
+        <v>2345365</v>
       </c>
       <c r="E16">
-        <v>0</v>
+        <v>2271623</v>
       </c>
       <c r="F16">
-        <v>120</v>
+        <v>4616988</v>
       </c>
       <c r="G16">
-        <v>1.47</v>
+        <v>413.3</v>
       </c>
       <c r="H16">
-        <v>10</v>
-      </c>
-      <c r="I16" t="str">
-        <v/>
+        <v>2</v>
+      </c>
+      <c r="I16">
+        <v>10960</v>
+      </c>
+      <c r="J16">
+        <v>5.82</v>
+      </c>
+      <c r="K16">
+        <v>638</v>
       </c>
     </row>
     <row r="17">
@@ -879,28 +978,34 @@
         <v>2026-02-16</v>
       </c>
       <c r="B17">
-        <v>5638766</v>
+        <v>27047244</v>
       </c>
       <c r="C17">
-        <v>52</v>
+        <v>225</v>
       </c>
       <c r="D17">
-        <v>1</v>
+        <v>2288974</v>
       </c>
       <c r="E17">
-        <v>48</v>
+        <v>3341964</v>
       </c>
       <c r="F17">
-        <v>6703</v>
+        <v>5630938</v>
       </c>
       <c r="G17">
-        <v>6.19</v>
+        <v>380.3</v>
       </c>
       <c r="H17">
-        <v>2489</v>
-      </c>
-      <c r="I17" t="str">
-        <v>facebook</v>
+        <v>2</v>
+      </c>
+      <c r="I17">
+        <v>14540</v>
+      </c>
+      <c r="J17">
+        <v>7.31</v>
+      </c>
+      <c r="K17">
+        <v>1063</v>
       </c>
     </row>
     <row r="18">
@@ -908,28 +1013,34 @@
         <v>2026-02-17</v>
       </c>
       <c r="B18">
-        <v>4818707</v>
+        <v>17303150</v>
       </c>
       <c r="C18">
-        <v>42</v>
+        <v>144</v>
       </c>
       <c r="D18">
-        <v>0</v>
+        <v>690756</v>
       </c>
       <c r="E18">
-        <v>0</v>
+        <v>2237155</v>
       </c>
       <c r="F18">
-        <v>365</v>
+        <v>2927911</v>
       </c>
       <c r="G18">
-        <v>0.67</v>
+        <v>491</v>
       </c>
       <c r="H18">
-        <v>9</v>
-      </c>
-      <c r="I18" t="str">
-        <v>instagram</v>
+        <v>2</v>
+      </c>
+      <c r="I18">
+        <v>11855</v>
+      </c>
+      <c r="J18">
+        <v>6.19</v>
+      </c>
+      <c r="K18">
+        <v>734</v>
       </c>
     </row>
     <row r="19">
@@ -937,28 +1048,34 @@
         <v>2026-02-18</v>
       </c>
       <c r="B19">
-        <v>6725620</v>
+        <v>29015748</v>
       </c>
       <c r="C19">
-        <v>69</v>
+        <v>242</v>
       </c>
       <c r="D19">
-        <v>1</v>
+        <v>3400842</v>
       </c>
       <c r="E19">
-        <v>49</v>
+        <v>2868387</v>
       </c>
       <c r="F19">
-        <v>4682</v>
+        <v>6269229</v>
       </c>
       <c r="G19">
-        <v>7.66</v>
+        <v>362.8</v>
       </c>
       <c r="H19">
-        <v>2152</v>
-      </c>
-      <c r="I19" t="str">
-        <v>both</v>
+        <v>2</v>
+      </c>
+      <c r="I19">
+        <v>12581</v>
+      </c>
+      <c r="J19">
+        <v>6.49</v>
+      </c>
+      <c r="K19">
+        <v>817</v>
       </c>
     </row>
     <row r="20">
@@ -966,28 +1083,34 @@
         <v>2026-02-19</v>
       </c>
       <c r="B20">
-        <v>4797537</v>
+        <v>16122047</v>
       </c>
       <c r="C20">
-        <v>43</v>
+        <v>134</v>
       </c>
       <c r="D20">
-        <v>0</v>
+        <v>948459</v>
       </c>
       <c r="E20">
-        <v>0</v>
+        <v>1703427</v>
       </c>
       <c r="F20">
-        <v>143</v>
+        <v>2651886</v>
       </c>
       <c r="G20">
-        <v>0.81</v>
+        <v>507.9</v>
       </c>
       <c r="H20">
-        <v>18</v>
-      </c>
-      <c r="I20" t="str">
-        <v>facebook</v>
+        <v>2</v>
+      </c>
+      <c r="I20">
+        <v>7960</v>
+      </c>
+      <c r="J20">
+        <v>4.57</v>
+      </c>
+      <c r="K20">
+        <v>364</v>
       </c>
     </row>
     <row r="21">
@@ -995,28 +1118,34 @@
         <v>2026-02-20</v>
       </c>
       <c r="B21">
-        <v>6166293</v>
+        <v>19370079</v>
       </c>
       <c r="C21">
-        <v>56</v>
+        <v>161</v>
       </c>
       <c r="D21">
-        <v>1</v>
+        <v>1735942</v>
       </c>
       <c r="E21">
-        <v>50</v>
+        <v>1701866</v>
       </c>
       <c r="F21">
-        <v>5006</v>
+        <v>3437808</v>
       </c>
       <c r="G21">
-        <v>5.5</v>
+        <v>463.4</v>
       </c>
       <c r="H21">
-        <v>826</v>
-      </c>
-      <c r="I21" t="str">
-        <v>instagram</v>
+        <v>2</v>
+      </c>
+      <c r="I21">
+        <v>8782</v>
+      </c>
+      <c r="J21">
+        <v>4.91</v>
+      </c>
+      <c r="K21">
+        <v>431</v>
       </c>
     </row>
     <row r="22">
@@ -1024,28 +1153,34 @@
         <v>2026-02-21</v>
       </c>
       <c r="B22">
-        <v>4950801</v>
+        <v>22716535</v>
       </c>
       <c r="C22">
-        <v>47</v>
+        <v>189</v>
       </c>
       <c r="D22">
-        <v>0</v>
+        <v>2457662</v>
       </c>
       <c r="E22">
-        <v>0</v>
+        <v>1878155</v>
       </c>
       <c r="F22">
-        <v>302</v>
+        <v>4335817</v>
       </c>
       <c r="G22">
-        <v>1.23</v>
+        <v>423.9</v>
       </c>
       <c r="H22">
-        <v>8</v>
-      </c>
-      <c r="I22" t="str">
-        <v/>
+        <v>2</v>
+      </c>
+      <c r="I22">
+        <v>9702</v>
+      </c>
+      <c r="J22">
+        <v>5.29</v>
+      </c>
+      <c r="K22">
+        <v>513</v>
       </c>
     </row>
     <row r="23">
@@ -1053,28 +1188,34 @@
         <v>2026-02-22</v>
       </c>
       <c r="B23">
-        <v>4746560</v>
+        <v>17303150</v>
       </c>
       <c r="C23">
-        <v>47</v>
+        <v>144</v>
       </c>
       <c r="D23">
-        <v>0</v>
+        <v>2569400</v>
       </c>
       <c r="E23">
-        <v>0</v>
+        <v>358511</v>
       </c>
       <c r="F23">
-        <v>132</v>
+        <v>2927911</v>
       </c>
       <c r="G23">
-        <v>1.77</v>
+        <v>491</v>
       </c>
       <c r="H23">
-        <v>9</v>
-      </c>
-      <c r="I23" t="str">
-        <v/>
+        <v>1</v>
+      </c>
+      <c r="I23">
+        <v>4234</v>
+      </c>
+      <c r="J23">
+        <v>3.01</v>
+      </c>
+      <c r="K23">
+        <v>127</v>
       </c>
     </row>
     <row r="24">
@@ -1082,28 +1223,34 @@
         <v>2026-02-23</v>
       </c>
       <c r="B24">
-        <v>5854461</v>
+        <v>10511811</v>
       </c>
       <c r="C24">
-        <v>52</v>
+        <v>88</v>
       </c>
       <c r="D24">
-        <v>1</v>
+        <v>178769</v>
       </c>
       <c r="E24">
-        <v>51</v>
+        <v>1314405</v>
       </c>
       <c r="F24">
-        <v>3583</v>
+        <v>1493174</v>
       </c>
       <c r="G24">
-        <v>6.96</v>
+        <v>604</v>
       </c>
       <c r="H24">
-        <v>1247</v>
-      </c>
-      <c r="I24" t="str">
-        <v>facebook</v>
+        <v>2</v>
+      </c>
+      <c r="I24">
+        <v>6847</v>
+      </c>
+      <c r="J24">
+        <v>4.1</v>
+      </c>
+      <c r="K24">
+        <v>281</v>
       </c>
     </row>
     <row r="25">
@@ -1111,28 +1258,34 @@
         <v>2026-02-24</v>
       </c>
       <c r="B25">
-        <v>5010033</v>
+        <v>20255906</v>
       </c>
       <c r="C25">
-        <v>52</v>
+        <v>169</v>
       </c>
       <c r="D25">
-        <v>0</v>
+        <v>2527008</v>
       </c>
       <c r="E25">
-        <v>0</v>
+        <v>1139789</v>
       </c>
       <c r="F25">
-        <v>120</v>
+        <v>3666797</v>
       </c>
       <c r="G25">
-        <v>0.63</v>
+        <v>452.4</v>
       </c>
       <c r="H25">
-        <v>12</v>
-      </c>
-      <c r="I25" t="str">
-        <v>instagram</v>
+        <v>2</v>
+      </c>
+      <c r="I25">
+        <v>7089</v>
+      </c>
+      <c r="J25">
+        <v>4.2</v>
+      </c>
+      <c r="K25">
+        <v>298</v>
       </c>
     </row>
     <row r="26">
@@ -1140,28 +1293,34 @@
         <v>2026-02-25</v>
       </c>
       <c r="B26">
-        <v>6397448</v>
+        <v>14547244</v>
       </c>
       <c r="C26">
-        <v>59</v>
+        <v>121</v>
       </c>
       <c r="D26">
-        <v>1</v>
+        <v>1025359</v>
       </c>
       <c r="E26">
-        <v>52</v>
+        <v>1275855</v>
       </c>
       <c r="F26">
-        <v>8660</v>
+        <v>2301214</v>
       </c>
       <c r="G26">
-        <v>4.27</v>
+        <v>532.2</v>
       </c>
       <c r="H26">
-        <v>1849</v>
-      </c>
-      <c r="I26" t="str">
-        <v>both</v>
+        <v>2</v>
+      </c>
+      <c r="I26">
+        <v>6048</v>
+      </c>
+      <c r="J26">
+        <v>3.77</v>
+      </c>
+      <c r="K26">
+        <v>228</v>
       </c>
     </row>
     <row r="27">
@@ -1169,28 +1328,34 @@
         <v>2026-02-26</v>
       </c>
       <c r="B27">
-        <v>4674438</v>
+        <v>16811024</v>
       </c>
       <c r="C27">
-        <v>47</v>
+        <v>140</v>
       </c>
       <c r="D27">
+        <v>2579463</v>
+      </c>
+      <c r="E27">
+        <v>232081</v>
+      </c>
+      <c r="F27">
+        <v>2811544</v>
+      </c>
+      <c r="G27">
+        <v>497.9</v>
+      </c>
+      <c r="H27">
         <v>0</v>
       </c>
-      <c r="E27">
-        <v>0</v>
-      </c>
-      <c r="F27">
-        <v>317</v>
-      </c>
-      <c r="G27">
-        <v>1.25</v>
-      </c>
-      <c r="H27">
-        <v>9</v>
-      </c>
-      <c r="I27" t="str">
-        <v>facebook</v>
+      <c r="I27">
+        <v>3847</v>
+      </c>
+      <c r="J27">
+        <v>2.85</v>
+      </c>
+      <c r="K27">
+        <v>110</v>
       </c>
     </row>
     <row r="28">
@@ -1198,28 +1363,34 @@
         <v>2026-02-27</v>
       </c>
       <c r="B28">
-        <v>6343275</v>
+        <v>19763780</v>
       </c>
       <c r="C28">
-        <v>60</v>
+        <v>165</v>
       </c>
       <c r="D28">
-        <v>1</v>
+        <v>1583896</v>
       </c>
       <c r="E28">
-        <v>53</v>
+        <v>1954910</v>
       </c>
       <c r="F28">
-        <v>5970</v>
+        <v>3538806</v>
       </c>
       <c r="G28">
-        <v>3.64</v>
+        <v>458.5</v>
       </c>
       <c r="H28">
-        <v>1087</v>
-      </c>
-      <c r="I28" t="str">
-        <v>instagram</v>
+        <v>2</v>
+      </c>
+      <c r="I28">
+        <v>10089</v>
+      </c>
+      <c r="J28">
+        <v>5.45</v>
+      </c>
+      <c r="K28">
+        <v>550</v>
       </c>
     </row>
     <row r="29">
@@ -1227,28 +1398,34 @@
         <v>2026-02-28</v>
       </c>
       <c r="B29">
-        <v>5706917</v>
+        <v>20649606</v>
       </c>
       <c r="C29">
-        <v>60</v>
+        <v>172</v>
       </c>
       <c r="D29">
-        <v>0</v>
+        <v>2647985</v>
       </c>
       <c r="E29">
-        <v>0</v>
+        <v>1122601</v>
       </c>
       <c r="F29">
-        <v>280</v>
+        <v>3770586</v>
       </c>
       <c r="G29">
-        <v>1.04</v>
+        <v>447.6</v>
       </c>
       <c r="H29">
-        <v>7</v>
-      </c>
-      <c r="I29" t="str">
-        <v/>
+        <v>2</v>
+      </c>
+      <c r="I29">
+        <v>7040</v>
+      </c>
+      <c r="J29">
+        <v>4.18</v>
+      </c>
+      <c r="K29">
+        <v>294</v>
       </c>
     </row>
     <row r="30">
@@ -1256,28 +1433,34 @@
         <v>2026-03-01</v>
       </c>
       <c r="B30">
-        <v>5087539</v>
+        <v>23602362</v>
       </c>
       <c r="C30">
-        <v>47</v>
+        <v>197</v>
       </c>
       <c r="D30">
-        <v>0</v>
+        <v>2769921</v>
       </c>
       <c r="E30">
-        <v>0</v>
+        <v>1818601</v>
       </c>
       <c r="F30">
-        <v>341</v>
+        <v>4588522</v>
       </c>
       <c r="G30">
-        <v>1.8</v>
+        <v>414.4</v>
       </c>
       <c r="H30">
-        <v>14</v>
-      </c>
-      <c r="I30" t="str">
-        <v/>
+        <v>2</v>
+      </c>
+      <c r="I30">
+        <v>9556</v>
+      </c>
+      <c r="J30">
+        <v>5.23</v>
+      </c>
+      <c r="K30">
+        <v>500</v>
       </c>
     </row>
     <row r="31">
@@ -1285,28 +1468,34 @@
         <v>2026-03-02</v>
       </c>
       <c r="B31">
-        <v>6614852</v>
+        <v>15334646</v>
       </c>
       <c r="C31">
-        <v>68</v>
+        <v>128</v>
       </c>
       <c r="D31">
-        <v>1</v>
+        <v>1038180</v>
       </c>
       <c r="E31">
-        <v>55</v>
+        <v>1435890</v>
       </c>
       <c r="F31">
-        <v>6373</v>
+        <v>2474070</v>
       </c>
       <c r="G31">
-        <v>4.3</v>
+        <v>519.8</v>
       </c>
       <c r="H31">
-        <v>822</v>
-      </c>
-      <c r="I31" t="str">
-        <v>facebook</v>
+        <v>2</v>
+      </c>
+      <c r="I31">
+        <v>6871</v>
+      </c>
+      <c r="J31">
+        <v>4.11</v>
+      </c>
+      <c r="K31">
+        <v>282</v>
       </c>
     </row>
     <row r="32">
@@ -1314,28 +1503,34 @@
         <v>2026-03-03</v>
       </c>
       <c r="B32">
-        <v>5901375</v>
+        <v>26062992</v>
       </c>
       <c r="C32">
-        <v>55</v>
+        <v>217</v>
       </c>
       <c r="D32">
-        <v>1</v>
+        <v>3365094</v>
       </c>
       <c r="E32">
-        <v>55</v>
+        <v>1958323</v>
       </c>
       <c r="F32">
-        <v>8014</v>
+        <v>5323417</v>
       </c>
       <c r="G32">
-        <v>4.65</v>
+        <v>389.6</v>
       </c>
       <c r="H32">
-        <v>1491</v>
-      </c>
-      <c r="I32" t="str">
-        <v>instagram</v>
+        <v>2</v>
+      </c>
+      <c r="I32">
+        <v>9847</v>
+      </c>
+      <c r="J32">
+        <v>5.35</v>
+      </c>
+      <c r="K32">
+        <v>527</v>
       </c>
     </row>
     <row r="33">
@@ -1343,28 +1538,34 @@
         <v>2026-03-04</v>
       </c>
       <c r="B33">
-        <v>6858984</v>
+        <v>16712598</v>
       </c>
       <c r="C33">
-        <v>67</v>
+        <v>139</v>
       </c>
       <c r="D33">
-        <v>1</v>
+        <v>1438642</v>
       </c>
       <c r="E33">
-        <v>56</v>
+        <v>1349862</v>
       </c>
       <c r="F33">
-        <v>8691</v>
+        <v>2788504</v>
       </c>
       <c r="G33">
-        <v>5.5</v>
+        <v>499.3</v>
       </c>
       <c r="H33">
-        <v>1434</v>
-      </c>
-      <c r="I33" t="str">
-        <v>both</v>
+        <v>2</v>
+      </c>
+      <c r="I33">
+        <v>7210</v>
+      </c>
+      <c r="J33">
+        <v>4.25</v>
+      </c>
+      <c r="K33">
+        <v>306</v>
       </c>
     </row>
     <row r="34">
@@ -1372,28 +1573,34 @@
         <v>2026-03-05</v>
       </c>
       <c r="B34">
-        <v>4978698</v>
+        <v>14448819</v>
       </c>
       <c r="C34">
-        <v>49</v>
+        <v>120</v>
       </c>
       <c r="D34">
+        <v>2032854</v>
+      </c>
+      <c r="E34">
+        <v>247101</v>
+      </c>
+      <c r="F34">
+        <v>2279955</v>
+      </c>
+      <c r="G34">
+        <v>533.7</v>
+      </c>
+      <c r="H34">
         <v>0</v>
       </c>
-      <c r="E34">
-        <v>0</v>
-      </c>
-      <c r="F34">
-        <v>130</v>
-      </c>
-      <c r="G34">
-        <v>0.61</v>
-      </c>
-      <c r="H34">
-        <v>1</v>
-      </c>
-      <c r="I34" t="str">
-        <v>facebook</v>
+      <c r="I34">
+        <v>3363</v>
+      </c>
+      <c r="J34">
+        <v>2.65</v>
+      </c>
+      <c r="K34">
+        <v>89</v>
       </c>
     </row>
     <row r="35">
@@ -1401,28 +1608,34 @@
         <v>2026-03-06</v>
       </c>
       <c r="B35">
-        <v>6600723</v>
+        <v>22125984</v>
       </c>
       <c r="C35">
-        <v>61</v>
+        <v>184</v>
       </c>
       <c r="D35">
-        <v>1</v>
+        <v>2863033</v>
       </c>
       <c r="E35">
-        <v>57</v>
+        <v>1307802</v>
       </c>
       <c r="F35">
-        <v>5746</v>
+        <v>4170835</v>
       </c>
       <c r="G35">
-        <v>5.17</v>
+        <v>430.5</v>
       </c>
       <c r="H35">
-        <v>1485</v>
-      </c>
-      <c r="I35" t="str">
-        <v>instagram</v>
+        <v>2</v>
+      </c>
+      <c r="I35">
+        <v>7839</v>
+      </c>
+      <c r="J35">
+        <v>4.52</v>
+      </c>
+      <c r="K35">
+        <v>354</v>
       </c>
     </row>
     <row r="36">
@@ -1430,28 +1643,34 @@
         <v>2026-03-07</v>
       </c>
       <c r="B36">
-        <v>5273541</v>
+        <v>14350394</v>
       </c>
       <c r="C36">
-        <v>52</v>
+        <v>120</v>
       </c>
       <c r="D36">
+        <v>2021685</v>
+      </c>
+      <c r="E36">
+        <v>237090</v>
+      </c>
+      <c r="F36">
+        <v>2258775</v>
+      </c>
+      <c r="G36">
+        <v>535.3</v>
+      </c>
+      <c r="H36">
         <v>0</v>
       </c>
-      <c r="E36">
-        <v>0</v>
-      </c>
-      <c r="F36">
-        <v>177</v>
-      </c>
-      <c r="G36">
-        <v>1.8</v>
-      </c>
-      <c r="H36">
-        <v>19</v>
-      </c>
-      <c r="I36" t="str">
-        <v/>
+      <c r="I36">
+        <v>3339</v>
+      </c>
+      <c r="J36">
+        <v>2.64</v>
+      </c>
+      <c r="K36">
+        <v>88</v>
       </c>
     </row>
     <row r="37">
@@ -1459,28 +1678,34 @@
         <v>2026-03-08</v>
       </c>
       <c r="B37">
-        <v>5208929</v>
+        <v>17598425</v>
       </c>
       <c r="C37">
-        <v>45</v>
+        <v>147</v>
       </c>
       <c r="D37">
+        <v>2742045</v>
+      </c>
+      <c r="E37">
+        <v>256616</v>
+      </c>
+      <c r="F37">
+        <v>2998661</v>
+      </c>
+      <c r="G37">
+        <v>486.9</v>
+      </c>
+      <c r="H37">
         <v>0</v>
       </c>
-      <c r="E37">
-        <v>0</v>
-      </c>
-      <c r="F37">
-        <v>176</v>
-      </c>
-      <c r="G37">
-        <v>1.33</v>
-      </c>
-      <c r="H37">
-        <v>4</v>
-      </c>
-      <c r="I37" t="str">
-        <v/>
+      <c r="I37">
+        <v>3992</v>
+      </c>
+      <c r="J37">
+        <v>2.91</v>
+      </c>
+      <c r="K37">
+        <v>116</v>
       </c>
     </row>
     <row r="38">
@@ -1488,28 +1713,34 @@
         <v>2026-03-09</v>
       </c>
       <c r="B38">
-        <v>6141719</v>
+        <v>30000000</v>
       </c>
       <c r="C38">
-        <v>56</v>
+        <v>250</v>
       </c>
       <c r="D38">
-        <v>1</v>
+        <v>3329290</v>
       </c>
       <c r="E38">
-        <v>58</v>
+        <v>3270710</v>
       </c>
       <c r="F38">
-        <v>3749</v>
+        <v>6600000</v>
       </c>
       <c r="G38">
-        <v>3.65</v>
+        <v>354.5</v>
       </c>
       <c r="H38">
-        <v>411</v>
-      </c>
-      <c r="I38" t="str">
-        <v>facebook</v>
+        <v>2</v>
+      </c>
+      <c r="I38">
+        <v>13597</v>
+      </c>
+      <c r="J38">
+        <v>6.92</v>
+      </c>
+      <c r="K38">
+        <v>941</v>
       </c>
     </row>
     <row r="39">
@@ -1517,28 +1748,34 @@
         <v>2026-03-10</v>
       </c>
       <c r="B39">
-        <v>7208287</v>
+        <v>19468504</v>
       </c>
       <c r="C39">
-        <v>71</v>
+        <v>162</v>
       </c>
       <c r="D39">
-        <v>1</v>
+        <v>699041</v>
       </c>
       <c r="E39">
-        <v>59</v>
+        <v>2763900</v>
       </c>
       <c r="F39">
-        <v>4095</v>
+        <v>3462941</v>
       </c>
       <c r="G39">
-        <v>3.49</v>
+        <v>462.2</v>
       </c>
       <c r="H39">
-        <v>1000</v>
-      </c>
-      <c r="I39" t="str">
-        <v>instagram</v>
+        <v>2</v>
+      </c>
+      <c r="I39">
+        <v>14952</v>
+      </c>
+      <c r="J39">
+        <v>7.48</v>
+      </c>
+      <c r="K39">
+        <v>1118</v>
       </c>
     </row>
     <row r="40">
@@ -1546,28 +1783,34 @@
         <v>2026-03-11</v>
       </c>
       <c r="B40">
-        <v>6844575</v>
+        <v>14940945</v>
       </c>
       <c r="C40">
-        <v>64</v>
+        <v>125</v>
       </c>
       <c r="D40">
-        <v>1</v>
+        <v>504112</v>
       </c>
       <c r="E40">
-        <v>59</v>
+        <v>1882910</v>
       </c>
       <c r="F40">
-        <v>6881</v>
+        <v>2387022</v>
       </c>
       <c r="G40">
-        <v>3.07</v>
+        <v>525.9</v>
       </c>
       <c r="H40">
-        <v>1267</v>
-      </c>
-      <c r="I40" t="str">
-        <v>both</v>
+        <v>2</v>
+      </c>
+      <c r="I40">
+        <v>9460</v>
+      </c>
+      <c r="J40">
+        <v>5.19</v>
+      </c>
+      <c r="K40">
+        <v>491</v>
       </c>
     </row>
     <row r="41">
@@ -1575,28 +1818,34 @@
         <v>2026-03-12</v>
       </c>
       <c r="B41">
-        <v>4987873</v>
+        <v>26161417</v>
       </c>
       <c r="C41">
-        <v>45</v>
+        <v>218</v>
       </c>
       <c r="D41">
-        <v>0</v>
+        <v>2688137</v>
       </c>
       <c r="E41">
-        <v>0</v>
+        <v>2665684</v>
       </c>
       <c r="F41">
-        <v>343</v>
+        <v>5353821</v>
       </c>
       <c r="G41">
-        <v>0.6</v>
+        <v>388.6</v>
       </c>
       <c r="H41">
-        <v>15</v>
-      </c>
-      <c r="I41" t="str">
-        <v>facebook</v>
+        <v>2</v>
+      </c>
+      <c r="I41">
+        <v>12121</v>
+      </c>
+      <c r="J41">
+        <v>6.3</v>
+      </c>
+      <c r="K41">
+        <v>764</v>
       </c>
     </row>
     <row r="42">
@@ -1604,28 +1853,34 @@
         <v>2026-03-13</v>
       </c>
       <c r="B42">
-        <v>5758482</v>
+        <v>21338583</v>
       </c>
       <c r="C42">
-        <v>54</v>
+        <v>178</v>
       </c>
       <c r="D42">
-        <v>1</v>
+        <v>2373558</v>
       </c>
       <c r="E42">
-        <v>60</v>
+        <v>1581641</v>
       </c>
       <c r="F42">
-        <v>5653</v>
+        <v>3955199</v>
       </c>
       <c r="G42">
-        <v>7.05</v>
+        <v>439.5</v>
       </c>
       <c r="H42">
-        <v>1993</v>
-      </c>
-      <c r="I42" t="str">
-        <v>instagram</v>
+        <v>2</v>
+      </c>
+      <c r="I42">
+        <v>8395</v>
+      </c>
+      <c r="J42">
+        <v>4.75</v>
+      </c>
+      <c r="K42">
+        <v>399</v>
       </c>
     </row>
     <row r="43">
@@ -1633,28 +1888,34 @@
         <v>2026-03-14</v>
       </c>
       <c r="B43">
-        <v>5666817</v>
+        <v>21830709</v>
       </c>
       <c r="C43">
-        <v>50</v>
+        <v>182</v>
       </c>
       <c r="D43">
-        <v>0</v>
+        <v>1916686</v>
       </c>
       <c r="E43">
-        <v>0</v>
+        <v>2172704</v>
       </c>
       <c r="F43">
-        <v>164</v>
+        <v>4089390</v>
       </c>
       <c r="G43">
-        <v>1.86</v>
+        <v>433.8</v>
       </c>
       <c r="H43">
-        <v>13</v>
-      </c>
-      <c r="I43" t="str">
-        <v/>
+        <v>2</v>
+      </c>
+      <c r="I43">
+        <v>11081</v>
+      </c>
+      <c r="J43">
+        <v>5.87</v>
+      </c>
+      <c r="K43">
+        <v>650</v>
       </c>
     </row>
     <row r="44">
@@ -1662,28 +1923,34 @@
         <v>2026-03-15</v>
       </c>
       <c r="B44">
-        <v>4603948</v>
+        <v>25374016</v>
       </c>
       <c r="C44">
-        <v>43</v>
+        <v>211</v>
       </c>
       <c r="D44">
-        <v>0</v>
+        <v>3259719</v>
       </c>
       <c r="E44">
-        <v>0</v>
+        <v>1853045</v>
       </c>
       <c r="F44">
-        <v>266</v>
+        <v>5112764</v>
       </c>
       <c r="G44">
-        <v>1.91</v>
+        <v>396.3</v>
       </c>
       <c r="H44">
-        <v>3</v>
-      </c>
-      <c r="I44" t="str">
-        <v/>
+        <v>2</v>
+      </c>
+      <c r="I44">
+        <v>9702</v>
+      </c>
+      <c r="J44">
+        <v>5.29</v>
+      </c>
+      <c r="K44">
+        <v>513</v>
       </c>
     </row>
     <row r="45">
@@ -1691,28 +1958,34 @@
         <v>2026-03-16</v>
       </c>
       <c r="B45">
-        <v>6651967</v>
+        <v>17696850</v>
       </c>
       <c r="C45">
-        <v>68</v>
+        <v>147</v>
       </c>
       <c r="D45">
+        <v>2409222</v>
+      </c>
+      <c r="E45">
+        <v>613177</v>
+      </c>
+      <c r="F45">
+        <v>3022399</v>
+      </c>
+      <c r="G45">
+        <v>485.5</v>
+      </c>
+      <c r="H45">
         <v>1</v>
       </c>
-      <c r="E45">
-        <v>62</v>
-      </c>
-      <c r="F45">
-        <v>5970</v>
-      </c>
-      <c r="G45">
-        <v>4.21</v>
-      </c>
-      <c r="H45">
-        <v>1257</v>
-      </c>
-      <c r="I45" t="str">
-        <v>facebook</v>
+      <c r="I45">
+        <v>5032</v>
+      </c>
+      <c r="J45">
+        <v>3.35</v>
+      </c>
+      <c r="K45">
+        <v>169</v>
       </c>
     </row>
     <row r="46">
@@ -1720,28 +1993,34 @@
         <v>2026-03-17</v>
       </c>
       <c r="B46">
-        <v>6988770</v>
+        <v>13366142</v>
       </c>
       <c r="C46">
-        <v>73</v>
+        <v>111</v>
       </c>
       <c r="D46">
-        <v>1</v>
+        <v>285773</v>
       </c>
       <c r="E46">
-        <v>62</v>
+        <v>1765456</v>
       </c>
       <c r="F46">
-        <v>6424</v>
+        <v>2051229</v>
       </c>
       <c r="G46">
-        <v>7.79</v>
+        <v>551.6</v>
       </c>
       <c r="H46">
-        <v>3003</v>
-      </c>
-      <c r="I46" t="str">
-        <v>instagram</v>
+        <v>2</v>
+      </c>
+      <c r="I46">
+        <v>9218</v>
+      </c>
+      <c r="J46">
+        <v>5.09</v>
+      </c>
+      <c r="K46">
+        <v>469</v>
       </c>
     </row>
     <row r="47">
@@ -1749,28 +2028,34 @@
         <v>2026-03-18</v>
       </c>
       <c r="B47">
-        <v>6555795</v>
+        <v>19665354</v>
       </c>
       <c r="C47">
-        <v>63</v>
+        <v>164</v>
       </c>
       <c r="D47">
-        <v>1</v>
+        <v>1976738</v>
       </c>
       <c r="E47">
-        <v>63</v>
+        <v>1536702</v>
       </c>
       <c r="F47">
-        <v>6384</v>
+        <v>3513440</v>
       </c>
       <c r="G47">
-        <v>3.8</v>
+        <v>459.7</v>
       </c>
       <c r="H47">
-        <v>1213</v>
-      </c>
-      <c r="I47" t="str">
-        <v>both</v>
+        <v>2</v>
+      </c>
+      <c r="I47">
+        <v>8444</v>
+      </c>
+      <c r="J47">
+        <v>4.77</v>
+      </c>
+      <c r="K47">
+        <v>403</v>
       </c>
     </row>
     <row r="48">
@@ -1778,28 +2063,34 @@
         <v>2026-03-19</v>
       </c>
       <c r="B48">
-        <v>4801269</v>
+        <v>15433071</v>
       </c>
       <c r="C48">
-        <v>46</v>
+        <v>129</v>
       </c>
       <c r="D48">
-        <v>0</v>
+        <v>1480409</v>
       </c>
       <c r="E48">
-        <v>0</v>
+        <v>1015617</v>
       </c>
       <c r="F48">
-        <v>317</v>
+        <v>2496026</v>
       </c>
       <c r="G48">
-        <v>1.89</v>
+        <v>518.3</v>
       </c>
       <c r="H48">
-        <v>19</v>
-      </c>
-      <c r="I48" t="str">
-        <v>facebook</v>
+        <v>2</v>
+      </c>
+      <c r="I48">
+        <v>5395</v>
+      </c>
+      <c r="J48">
+        <v>3.5</v>
+      </c>
+      <c r="K48">
+        <v>189</v>
       </c>
     </row>
     <row r="49">
@@ -1807,28 +2098,34 @@
         <v>2026-03-20</v>
       </c>
       <c r="B49">
-        <v>6040075</v>
+        <v>27834646</v>
       </c>
       <c r="C49">
-        <v>58</v>
+        <v>232</v>
       </c>
       <c r="D49">
-        <v>1</v>
+        <v>2888948</v>
       </c>
       <c r="E49">
-        <v>64</v>
+        <v>2993587</v>
       </c>
       <c r="F49">
-        <v>8695</v>
+        <v>5882535</v>
       </c>
       <c r="G49">
-        <v>7.36</v>
+        <v>373.2</v>
       </c>
       <c r="H49">
-        <v>4480</v>
-      </c>
-      <c r="I49" t="str">
-        <v>instagram</v>
+        <v>2</v>
+      </c>
+      <c r="I49">
+        <v>13040</v>
+      </c>
+      <c r="J49">
+        <v>6.68</v>
+      </c>
+      <c r="K49">
+        <v>871</v>
       </c>
     </row>
     <row r="50">
@@ -1836,28 +2133,34 @@
         <v>2026-03-21</v>
       </c>
       <c r="B50">
-        <v>5399890</v>
+        <v>19566929</v>
       </c>
       <c r="C50">
-        <v>52</v>
+        <v>163</v>
       </c>
       <c r="D50">
-        <v>0</v>
+        <v>2448569</v>
       </c>
       <c r="E50">
-        <v>0</v>
+        <v>1039583</v>
       </c>
       <c r="F50">
-        <v>220</v>
+        <v>3488152</v>
       </c>
       <c r="G50">
-        <v>1.14</v>
+        <v>461</v>
       </c>
       <c r="H50">
-        <v>18</v>
-      </c>
-      <c r="I50" t="str">
-        <v/>
+        <v>2</v>
+      </c>
+      <c r="I50">
+        <v>6823</v>
+      </c>
+      <c r="J50">
+        <v>4.09</v>
+      </c>
+      <c r="K50">
+        <v>279</v>
       </c>
     </row>
     <row r="51">
@@ -1865,28 +2168,34 @@
         <v>2026-03-22</v>
       </c>
       <c r="B51">
-        <v>4860727</v>
+        <v>14547244</v>
       </c>
       <c r="C51">
-        <v>48</v>
+        <v>121</v>
       </c>
       <c r="D51">
-        <v>0</v>
+        <v>1106827</v>
       </c>
       <c r="E51">
-        <v>0</v>
+        <v>1194387</v>
       </c>
       <c r="F51">
-        <v>393</v>
+        <v>2301214</v>
       </c>
       <c r="G51">
-        <v>1.18</v>
+        <v>532.2</v>
       </c>
       <c r="H51">
-        <v>10</v>
-      </c>
-      <c r="I51" t="str">
-        <v/>
+        <v>2</v>
+      </c>
+      <c r="I51">
+        <v>5831</v>
+      </c>
+      <c r="J51">
+        <v>3.68</v>
+      </c>
+      <c r="K51">
+        <v>215</v>
       </c>
     </row>
     <row r="52">
@@ -1894,28 +2203,34 @@
         <v>2026-03-23</v>
       </c>
       <c r="B52">
-        <v>7391873</v>
+        <v>16220472</v>
       </c>
       <c r="C52">
-        <v>70</v>
+        <v>135</v>
       </c>
       <c r="D52">
-        <v>1</v>
+        <v>2416967</v>
       </c>
       <c r="E52">
-        <v>65</v>
+        <v>257495</v>
       </c>
       <c r="F52">
-        <v>5298</v>
+        <v>2674462</v>
       </c>
       <c r="G52">
-        <v>7.13</v>
+        <v>506.5</v>
       </c>
       <c r="H52">
-        <v>1133</v>
-      </c>
-      <c r="I52" t="str">
-        <v>facebook</v>
+        <v>0</v>
+      </c>
+      <c r="I52">
+        <v>3750</v>
+      </c>
+      <c r="J52">
+        <v>2.81</v>
+      </c>
+      <c r="K52">
+        <v>105</v>
       </c>
     </row>
     <row r="53">
@@ -1923,28 +2238,34 @@
         <v>2026-03-24</v>
       </c>
       <c r="B53">
-        <v>6852433</v>
+        <v>15531496</v>
       </c>
       <c r="C53">
-        <v>62</v>
+        <v>129</v>
       </c>
       <c r="D53">
-        <v>1</v>
+        <v>1578486</v>
       </c>
       <c r="E53">
-        <v>66</v>
+        <v>939573</v>
       </c>
       <c r="F53">
-        <v>8942</v>
+        <v>2518059</v>
       </c>
       <c r="G53">
-        <v>6.74</v>
+        <v>516.8</v>
       </c>
       <c r="H53">
-        <v>3616</v>
-      </c>
-      <c r="I53" t="str">
-        <v>instagram</v>
+        <v>2</v>
+      </c>
+      <c r="I53">
+        <v>5323</v>
+      </c>
+      <c r="J53">
+        <v>3.47</v>
+      </c>
+      <c r="K53">
+        <v>185</v>
       </c>
     </row>
     <row r="54">
@@ -1952,28 +2273,34 @@
         <v>2026-03-25</v>
       </c>
       <c r="B54">
-        <v>7115994</v>
+        <v>27244094</v>
       </c>
       <c r="C54">
-        <v>65</v>
+        <v>227</v>
       </c>
       <c r="D54">
-        <v>1</v>
+        <v>2642893</v>
       </c>
       <c r="E54">
-        <v>66</v>
+        <v>3050479</v>
       </c>
       <c r="F54">
-        <v>7837</v>
+        <v>5693372</v>
       </c>
       <c r="G54">
-        <v>3.51</v>
+        <v>378.5</v>
       </c>
       <c r="H54">
-        <v>1100</v>
-      </c>
-      <c r="I54" t="str">
-        <v>both</v>
+        <v>2</v>
+      </c>
+      <c r="I54">
+        <v>13089</v>
+      </c>
+      <c r="J54">
+        <v>6.7</v>
+      </c>
+      <c r="K54">
+        <v>877</v>
       </c>
     </row>
     <row r="55">
@@ -1981,28 +2308,34 @@
         <v>2026-03-26</v>
       </c>
       <c r="B55">
-        <v>5119267</v>
+        <v>25866142</v>
       </c>
       <c r="C55">
-        <v>45</v>
+        <v>216</v>
       </c>
       <c r="D55">
-        <v>0</v>
+        <v>2093625</v>
       </c>
       <c r="E55">
-        <v>0</v>
+        <v>3169218</v>
       </c>
       <c r="F55">
-        <v>353</v>
+        <v>5262843</v>
       </c>
       <c r="G55">
-        <v>1.27</v>
+        <v>391.5</v>
       </c>
       <c r="H55">
-        <v>12</v>
-      </c>
-      <c r="I55" t="str">
-        <v>facebook</v>
+        <v>2</v>
+      </c>
+      <c r="I55">
+        <v>14177</v>
+      </c>
+      <c r="J55">
+        <v>7.16</v>
+      </c>
+      <c r="K55">
+        <v>1015</v>
       </c>
     </row>
     <row r="56">
@@ -2010,28 +2343,34 @@
         <v>2026-03-27</v>
       </c>
       <c r="B56">
-        <v>6734716</v>
+        <v>24881890</v>
       </c>
       <c r="C56">
-        <v>65</v>
+        <v>207</v>
       </c>
       <c r="D56">
-        <v>1</v>
+        <v>2990521</v>
       </c>
       <c r="E56">
-        <v>67</v>
+        <v>1974102</v>
       </c>
       <c r="F56">
-        <v>4997</v>
+        <v>4964623</v>
       </c>
       <c r="G56">
-        <v>5.64</v>
+        <v>401.2</v>
       </c>
       <c r="H56">
-        <v>1127</v>
-      </c>
-      <c r="I56" t="str">
-        <v>instagram</v>
+        <v>2</v>
+      </c>
+      <c r="I56">
+        <v>9968</v>
+      </c>
+      <c r="J56">
+        <v>5.4</v>
+      </c>
+      <c r="K56">
+        <v>538</v>
       </c>
     </row>
     <row r="57">
@@ -2039,28 +2378,34 @@
         <v>2026-03-28</v>
       </c>
       <c r="B57">
-        <v>5228319</v>
+        <v>28326772</v>
       </c>
       <c r="C57">
-        <v>49</v>
+        <v>236</v>
       </c>
       <c r="D57">
-        <v>0</v>
+        <v>2431580</v>
       </c>
       <c r="E57">
-        <v>0</v>
+        <v>3610721</v>
       </c>
       <c r="F57">
-        <v>393</v>
+        <v>6042301</v>
       </c>
       <c r="G57">
-        <v>1.94</v>
+        <v>368.8</v>
       </c>
       <c r="H57">
-        <v>9</v>
-      </c>
-      <c r="I57" t="str">
-        <v/>
+        <v>2</v>
+      </c>
+      <c r="I57">
+        <v>14952</v>
+      </c>
+      <c r="J57">
+        <v>7.48</v>
+      </c>
+      <c r="K57">
+        <v>1118</v>
       </c>
     </row>
     <row r="58">
@@ -2068,28 +2413,34 @@
         <v>2026-03-29</v>
       </c>
       <c r="B58">
-        <v>5494607</v>
+        <v>10413386</v>
       </c>
       <c r="C58">
-        <v>55</v>
+        <v>87</v>
       </c>
       <c r="D58">
-        <v>0</v>
+        <v>60985</v>
       </c>
       <c r="E58">
-        <v>0</v>
+        <v>1414108</v>
       </c>
       <c r="F58">
-        <v>368</v>
+        <v>1475093</v>
       </c>
       <c r="G58">
-        <v>1.49</v>
+        <v>605.9</v>
       </c>
       <c r="H58">
-        <v>1</v>
-      </c>
-      <c r="I58" t="str">
-        <v/>
+        <v>2</v>
+      </c>
+      <c r="I58">
+        <v>9798</v>
+      </c>
+      <c r="J58">
+        <v>5.33</v>
+      </c>
+      <c r="K58">
+        <v>522</v>
       </c>
     </row>
     <row r="59">
@@ -2097,28 +2448,34 @@
         <v>2026-03-30</v>
       </c>
       <c r="B59">
-        <v>7267955</v>
+        <v>17992126</v>
       </c>
       <c r="C59">
-        <v>76</v>
+        <v>150</v>
       </c>
       <c r="D59">
-        <v>1</v>
+        <v>1667066</v>
       </c>
       <c r="E59">
-        <v>69</v>
+        <v>1427013</v>
       </c>
       <c r="F59">
-        <v>8288</v>
+        <v>3094079</v>
       </c>
       <c r="G59">
-        <v>3.36</v>
+        <v>481.5</v>
       </c>
       <c r="H59">
-        <v>1949</v>
-      </c>
-      <c r="I59" t="str">
-        <v>facebook</v>
+        <v>2</v>
+      </c>
+      <c r="I59">
+        <v>7645</v>
+      </c>
+      <c r="J59">
+        <v>4.44</v>
+      </c>
+      <c r="K59">
+        <v>339</v>
       </c>
     </row>
     <row r="60">
@@ -2126,28 +2483,34 @@
         <v>2026-03-31</v>
       </c>
       <c r="B60">
-        <v>6718255</v>
+        <v>28425197</v>
       </c>
       <c r="C60">
-        <v>69</v>
+        <v>237</v>
       </c>
       <c r="D60">
-        <v>1</v>
+        <v>2523972</v>
       </c>
       <c r="E60">
-        <v>69</v>
+        <v>3550515</v>
       </c>
       <c r="F60">
-        <v>5924</v>
+        <v>6074487</v>
       </c>
       <c r="G60">
-        <v>4.24</v>
+        <v>367.9</v>
       </c>
       <c r="H60">
-        <v>1507</v>
-      </c>
-      <c r="I60" t="str">
-        <v>instagram</v>
+        <v>2</v>
+      </c>
+      <c r="I60">
+        <v>15000</v>
+      </c>
+      <c r="J60">
+        <v>7.5</v>
+      </c>
+      <c r="K60">
+        <v>1125</v>
       </c>
     </row>
     <row r="61">
@@ -2155,28 +2518,34 @@
         <v>2026-04-01</v>
       </c>
       <c r="B61">
-        <v>6014210</v>
+        <v>23110236</v>
       </c>
       <c r="C61">
-        <v>53</v>
+        <v>193</v>
       </c>
       <c r="D61">
-        <v>1</v>
+        <v>2413499</v>
       </c>
       <c r="E61">
-        <v>70</v>
+        <v>2033857</v>
       </c>
       <c r="F61">
-        <v>7791</v>
+        <v>4447356</v>
       </c>
       <c r="G61">
-        <v>6.87</v>
+        <v>419.6</v>
       </c>
       <c r="H61">
-        <v>1606</v>
-      </c>
-      <c r="I61" t="str">
-        <v>both</v>
+        <v>2</v>
+      </c>
+      <c r="I61">
+        <v>10137</v>
+      </c>
+      <c r="J61">
+        <v>5.47</v>
+      </c>
+      <c r="K61">
+        <v>554</v>
       </c>
     </row>
     <row r="62">
@@ -2184,28 +2553,34 @@
         <v>2026-04-02</v>
       </c>
       <c r="B62">
-        <v>6276909</v>
+        <v>12972441</v>
       </c>
       <c r="C62">
-        <v>62</v>
+        <v>108</v>
       </c>
       <c r="D62">
+        <v>1543989</v>
+      </c>
+      <c r="E62">
+        <v>426392</v>
+      </c>
+      <c r="F62">
+        <v>1970381</v>
+      </c>
+      <c r="G62">
+        <v>558.4</v>
+      </c>
+      <c r="H62">
         <v>1</v>
       </c>
-      <c r="E62">
-        <v>70</v>
-      </c>
-      <c r="F62">
-        <v>4538</v>
-      </c>
-      <c r="G62">
-        <v>6.42</v>
-      </c>
-      <c r="H62">
-        <v>874</v>
-      </c>
-      <c r="I62" t="str">
-        <v>facebook</v>
+      <c r="I62">
+        <v>3484</v>
+      </c>
+      <c r="J62">
+        <v>2.7</v>
+      </c>
+      <c r="K62">
+        <v>94</v>
       </c>
     </row>
     <row r="63">
@@ -2213,28 +2588,34 @@
         <v>2026-04-03</v>
       </c>
       <c r="B63">
-        <v>6721024</v>
+        <v>28818898</v>
       </c>
       <c r="C63">
-        <v>65</v>
+        <v>240</v>
       </c>
       <c r="D63">
-        <v>1</v>
+        <v>3135648</v>
       </c>
       <c r="E63">
-        <v>71</v>
+        <v>3068357</v>
       </c>
       <c r="F63">
-        <v>4642</v>
+        <v>6204005</v>
       </c>
       <c r="G63">
-        <v>6.61</v>
+        <v>364.5</v>
       </c>
       <c r="H63">
-        <v>1534</v>
-      </c>
-      <c r="I63" t="str">
-        <v>instagram</v>
+        <v>2</v>
+      </c>
+      <c r="I63">
+        <v>13331</v>
+      </c>
+      <c r="J63">
+        <v>6.8</v>
+      </c>
+      <c r="K63">
+        <v>907</v>
       </c>
     </row>
     <row r="64">
@@ -2242,28 +2623,34 @@
         <v>2026-04-04</v>
       </c>
       <c r="B64">
-        <v>5204416</v>
+        <v>20452756</v>
       </c>
       <c r="C64">
-        <v>47</v>
+        <v>170</v>
       </c>
       <c r="D64">
-        <v>0</v>
+        <v>2664321</v>
       </c>
       <c r="E64">
-        <v>0</v>
+        <v>1054216</v>
       </c>
       <c r="F64">
-        <v>165</v>
+        <v>3718537</v>
       </c>
       <c r="G64">
-        <v>1.14</v>
+        <v>450</v>
       </c>
       <c r="H64">
-        <v>0</v>
-      </c>
-      <c r="I64" t="str">
-        <v/>
+        <v>2</v>
+      </c>
+      <c r="I64">
+        <v>6750</v>
+      </c>
+      <c r="J64">
+        <v>4.06</v>
+      </c>
+      <c r="K64">
+        <v>274</v>
       </c>
     </row>
     <row r="65">
@@ -2271,28 +2658,34 @@
         <v>2026-04-05</v>
       </c>
       <c r="B65">
-        <v>5497416</v>
+        <v>18779528</v>
       </c>
       <c r="C65">
-        <v>53</v>
+        <v>156</v>
       </c>
       <c r="D65">
-        <v>0</v>
+        <v>1202578</v>
       </c>
       <c r="E65">
-        <v>0</v>
+        <v>2086057</v>
       </c>
       <c r="F65">
-        <v>345</v>
+        <v>3288635</v>
       </c>
       <c r="G65">
-        <v>1.77</v>
+        <v>471</v>
       </c>
       <c r="H65">
-        <v>16</v>
-      </c>
-      <c r="I65" t="str">
-        <v/>
+        <v>2</v>
+      </c>
+      <c r="I65">
+        <v>10161</v>
+      </c>
+      <c r="J65">
+        <v>5.48</v>
+      </c>
+      <c r="K65">
+        <v>557</v>
       </c>
     </row>
     <row r="66">
@@ -2300,28 +2693,34 @@
         <v>2026-04-06</v>
       </c>
       <c r="B66">
-        <v>6983401</v>
+        <v>22716535</v>
       </c>
       <c r="C66">
-        <v>63</v>
+        <v>189</v>
       </c>
       <c r="D66">
-        <v>1</v>
+        <v>1467343</v>
       </c>
       <c r="E66">
-        <v>72</v>
+        <v>2868474</v>
       </c>
       <c r="F66">
-        <v>4537</v>
+        <v>4335817</v>
       </c>
       <c r="G66">
-        <v>4.46</v>
+        <v>423.9</v>
       </c>
       <c r="H66">
-        <v>809</v>
-      </c>
-      <c r="I66" t="str">
-        <v>facebook</v>
+        <v>2</v>
+      </c>
+      <c r="I66">
+        <v>13355</v>
+      </c>
+      <c r="J66">
+        <v>6.81</v>
+      </c>
+      <c r="K66">
+        <v>909</v>
       </c>
     </row>
     <row r="67">
@@ -2329,28 +2728,34 @@
         <v>2026-04-07</v>
       </c>
       <c r="B67">
-        <v>6475996</v>
+        <v>14153543</v>
       </c>
       <c r="C67">
-        <v>68</v>
+        <v>118</v>
       </c>
       <c r="D67">
-        <v>1</v>
+        <v>1204452</v>
       </c>
       <c r="E67">
-        <v>73</v>
+        <v>1012193</v>
       </c>
       <c r="F67">
-        <v>7572</v>
+        <v>2216645</v>
       </c>
       <c r="G67">
-        <v>7.89</v>
+        <v>538.5</v>
       </c>
       <c r="H67">
-        <v>1792</v>
-      </c>
-      <c r="I67" t="str">
-        <v>instagram</v>
+        <v>2</v>
+      </c>
+      <c r="I67">
+        <v>5250</v>
+      </c>
+      <c r="J67">
+        <v>3.44</v>
+      </c>
+      <c r="K67">
+        <v>181</v>
       </c>
     </row>
     <row r="68">
@@ -2358,28 +2763,34 @@
         <v>2026-04-08</v>
       </c>
       <c r="B68">
-        <v>6202488</v>
+        <v>14350394</v>
       </c>
       <c r="C68">
-        <v>64</v>
+        <v>120</v>
       </c>
       <c r="D68">
-        <v>1</v>
+        <v>395171</v>
       </c>
       <c r="E68">
-        <v>73</v>
+        <v>1863604</v>
       </c>
       <c r="F68">
-        <v>5847</v>
+        <v>2258775</v>
       </c>
       <c r="G68">
-        <v>4.3</v>
+        <v>535.3</v>
       </c>
       <c r="H68">
-        <v>1509</v>
-      </c>
-      <c r="I68" t="str">
-        <v>both</v>
+        <v>2</v>
+      </c>
+      <c r="I68">
+        <v>8952</v>
+      </c>
+      <c r="J68">
+        <v>4.98</v>
+      </c>
+      <c r="K68">
+        <v>446</v>
       </c>
     </row>
     <row r="69">
@@ -2387,28 +2798,34 @@
         <v>2026-04-09</v>
       </c>
       <c r="B69">
-        <v>6984559</v>
+        <v>18188976</v>
       </c>
       <c r="C69">
-        <v>67</v>
+        <v>152</v>
       </c>
       <c r="D69">
-        <v>1</v>
+        <v>1919245</v>
       </c>
       <c r="E69">
-        <v>74</v>
+        <v>1223008</v>
       </c>
       <c r="F69">
-        <v>8702</v>
+        <v>3142253</v>
       </c>
       <c r="G69">
-        <v>4.3</v>
+        <v>478.9</v>
       </c>
       <c r="H69">
-        <v>2245</v>
-      </c>
-      <c r="I69" t="str">
-        <v>facebook</v>
+        <v>2</v>
+      </c>
+      <c r="I69">
+        <v>6508</v>
+      </c>
+      <c r="J69">
+        <v>3.96</v>
+      </c>
+      <c r="K69">
+        <v>258</v>
       </c>
     </row>
     <row r="70">
@@ -2416,28 +2833,34 @@
         <v>2026-04-10</v>
       </c>
       <c r="B70">
-        <v>7293308</v>
+        <v>23602362</v>
       </c>
       <c r="C70">
-        <v>66</v>
+        <v>197</v>
       </c>
       <c r="D70">
-        <v>1</v>
+        <v>2702222</v>
       </c>
       <c r="E70">
-        <v>74</v>
+        <v>1886300</v>
       </c>
       <c r="F70">
-        <v>4745</v>
+        <v>4588522</v>
       </c>
       <c r="G70">
-        <v>7.11</v>
+        <v>414.4</v>
       </c>
       <c r="H70">
-        <v>2024</v>
-      </c>
-      <c r="I70" t="str">
-        <v>instagram</v>
+        <v>2</v>
+      </c>
+      <c r="I70">
+        <v>9653</v>
+      </c>
+      <c r="J70">
+        <v>5.27</v>
+      </c>
+      <c r="K70">
+        <v>509</v>
       </c>
     </row>
     <row r="71">
@@ -2445,28 +2868,34 @@
         <v>2026-04-11</v>
       </c>
       <c r="B71">
-        <v>5153606</v>
+        <v>26948819</v>
       </c>
       <c r="C71">
-        <v>53</v>
+        <v>225</v>
       </c>
       <c r="D71">
-        <v>0</v>
+        <v>2531392</v>
       </c>
       <c r="E71">
-        <v>0</v>
+        <v>3068445</v>
       </c>
       <c r="F71">
-        <v>326</v>
+        <v>5599837</v>
       </c>
       <c r="G71">
-        <v>0.52</v>
+        <v>381.2</v>
       </c>
       <c r="H71">
-        <v>18</v>
-      </c>
-      <c r="I71" t="str">
-        <v/>
+        <v>2</v>
+      </c>
+      <c r="I71">
+        <v>13621</v>
+      </c>
+      <c r="J71">
+        <v>6.93</v>
+      </c>
+      <c r="K71">
+        <v>944</v>
       </c>
     </row>
     <row r="72">
@@ -2474,28 +2903,34 @@
         <v>2026-04-12</v>
       </c>
       <c r="B72">
-        <v>5052599</v>
+        <v>23011811</v>
       </c>
       <c r="C72">
-        <v>52</v>
+        <v>192</v>
       </c>
       <c r="D72">
-        <v>0</v>
+        <v>2296363</v>
       </c>
       <c r="E72">
-        <v>0</v>
+        <v>2122992</v>
       </c>
       <c r="F72">
-        <v>213</v>
+        <v>4419355</v>
       </c>
       <c r="G72">
-        <v>1.32</v>
+        <v>420.7</v>
       </c>
       <c r="H72">
-        <v>20</v>
-      </c>
-      <c r="I72" t="str">
-        <v/>
+        <v>2</v>
+      </c>
+      <c r="I72">
+        <v>10403</v>
+      </c>
+      <c r="J72">
+        <v>5.58</v>
+      </c>
+      <c r="K72">
+        <v>580</v>
       </c>
     </row>
     <row r="73">
@@ -2503,28 +2938,34 @@
         <v>2026-04-13</v>
       </c>
       <c r="B73">
-        <v>6790099</v>
+        <v>17204724</v>
       </c>
       <c r="C73">
-        <v>71</v>
+        <v>143</v>
       </c>
       <c r="D73">
-        <v>1</v>
+        <v>1615704</v>
       </c>
       <c r="E73">
-        <v>76</v>
+        <v>1288779</v>
       </c>
       <c r="F73">
-        <v>7231</v>
+        <v>2904483</v>
       </c>
       <c r="G73">
-        <v>7.19</v>
+        <v>492.4</v>
       </c>
       <c r="H73">
-        <v>3119</v>
-      </c>
-      <c r="I73" t="str">
-        <v>facebook</v>
+        <v>2</v>
+      </c>
+      <c r="I73">
+        <v>6460</v>
+      </c>
+      <c r="J73">
+        <v>3.94</v>
+      </c>
+      <c r="K73">
+        <v>255</v>
       </c>
     </row>
     <row r="74">
@@ -2532,28 +2973,34 @@
         <v>2026-04-14</v>
       </c>
       <c r="B74">
-        <v>6558020</v>
+        <v>13661417</v>
       </c>
       <c r="C74">
-        <v>68</v>
+        <v>114</v>
       </c>
       <c r="D74">
-        <v>1</v>
+        <v>251560</v>
       </c>
       <c r="E74">
-        <v>76</v>
+        <v>1861119</v>
       </c>
       <c r="F74">
-        <v>9801</v>
+        <v>2112679</v>
       </c>
       <c r="G74">
-        <v>4.46</v>
+        <v>546.6</v>
       </c>
       <c r="H74">
-        <v>2623</v>
-      </c>
-      <c r="I74" t="str">
-        <v>instagram</v>
+        <v>2</v>
+      </c>
+      <c r="I74">
+        <v>10984</v>
+      </c>
+      <c r="J74">
+        <v>5.83</v>
+      </c>
+      <c r="K74">
+        <v>640</v>
       </c>
     </row>
     <row r="75">
@@ -2561,28 +3008,34 @@
         <v>2026-04-15</v>
       </c>
       <c r="B75">
-        <v>7333663</v>
+        <v>15826772</v>
       </c>
       <c r="C75">
-        <v>76</v>
+        <v>132</v>
       </c>
       <c r="D75">
+        <v>2013835</v>
+      </c>
+      <c r="E75">
+        <v>570789</v>
+      </c>
+      <c r="F75">
+        <v>2584624</v>
+      </c>
+      <c r="G75">
+        <v>512.3</v>
+      </c>
+      <c r="H75">
         <v>1</v>
       </c>
-      <c r="E75">
-        <v>77</v>
-      </c>
-      <c r="F75">
-        <v>4975</v>
-      </c>
-      <c r="G75">
-        <v>6.31</v>
-      </c>
-      <c r="H75">
-        <v>2197</v>
-      </c>
-      <c r="I75" t="str">
-        <v>both</v>
+      <c r="I75">
+        <v>4379</v>
+      </c>
+      <c r="J75">
+        <v>3.07</v>
+      </c>
+      <c r="K75">
+        <v>134</v>
       </c>
     </row>
     <row r="76">
@@ -2590,28 +3043,34 @@
         <v>2026-04-16</v>
       </c>
       <c r="B76">
-        <v>7055537</v>
+        <v>21732283</v>
       </c>
       <c r="C76">
-        <v>73</v>
+        <v>181</v>
       </c>
       <c r="D76">
-        <v>1</v>
+        <v>2395111</v>
       </c>
       <c r="E76">
-        <v>77</v>
+        <v>1667286</v>
       </c>
       <c r="F76">
-        <v>7645</v>
+        <v>4062397</v>
       </c>
       <c r="G76">
-        <v>4.83</v>
+        <v>435</v>
       </c>
       <c r="H76">
-        <v>2216</v>
-      </c>
-      <c r="I76" t="str">
-        <v>facebook</v>
+        <v>2</v>
+      </c>
+      <c r="I76">
+        <v>8952</v>
+      </c>
+      <c r="J76">
+        <v>4.98</v>
+      </c>
+      <c r="K76">
+        <v>446</v>
       </c>
     </row>
     <row r="77">
@@ -2619,28 +3078,34 @@
         <v>2026-04-17</v>
       </c>
       <c r="B77">
-        <v>6623717</v>
+        <v>13562992</v>
       </c>
       <c r="C77">
-        <v>62</v>
+        <v>113</v>
       </c>
       <c r="D77">
-        <v>1</v>
+        <v>126949</v>
       </c>
       <c r="E77">
-        <v>78</v>
+        <v>1965169</v>
       </c>
       <c r="F77">
-        <v>4950</v>
+        <v>2092118</v>
       </c>
       <c r="G77">
-        <v>5.72</v>
+        <v>548.3</v>
       </c>
       <c r="H77">
-        <v>1699</v>
-      </c>
-      <c r="I77" t="str">
-        <v>instagram</v>
+        <v>2</v>
+      </c>
+      <c r="I77">
+        <v>13573</v>
+      </c>
+      <c r="J77">
+        <v>6.91</v>
+      </c>
+      <c r="K77">
+        <v>938</v>
       </c>
     </row>
     <row r="78">
@@ -2648,28 +3113,34 @@
         <v>2026-04-18</v>
       </c>
       <c r="B78">
-        <v>5245600</v>
+        <v>11791339</v>
       </c>
       <c r="C78">
-        <v>47</v>
+        <v>98</v>
       </c>
       <c r="D78">
-        <v>0</v>
+        <v>1195784</v>
       </c>
       <c r="E78">
-        <v>0</v>
+        <v>539493</v>
       </c>
       <c r="F78">
-        <v>229</v>
+        <v>1735277</v>
       </c>
       <c r="G78">
-        <v>1.53</v>
+        <v>579.5</v>
       </c>
       <c r="H78">
-        <v>16</v>
-      </c>
-      <c r="I78" t="str">
-        <v/>
+        <v>1</v>
+      </c>
+      <c r="I78">
+        <v>3387</v>
+      </c>
+      <c r="J78">
+        <v>2.66</v>
+      </c>
+      <c r="K78">
+        <v>90</v>
       </c>
     </row>
     <row r="79">
@@ -2677,28 +3148,34 @@
         <v>2026-04-19</v>
       </c>
       <c r="B79">
-        <v>5653695</v>
+        <v>18976378</v>
       </c>
       <c r="C79">
-        <v>54</v>
+        <v>158</v>
       </c>
       <c r="D79">
-        <v>0</v>
+        <v>1376868</v>
       </c>
       <c r="E79">
-        <v>0</v>
+        <v>1961181</v>
       </c>
       <c r="F79">
-        <v>295</v>
+        <v>3338049</v>
       </c>
       <c r="G79">
-        <v>1.65</v>
+        <v>468.5</v>
       </c>
       <c r="H79">
-        <v>18</v>
-      </c>
-      <c r="I79" t="str">
-        <v/>
+        <v>2</v>
+      </c>
+      <c r="I79">
+        <v>9895</v>
+      </c>
+      <c r="J79">
+        <v>5.37</v>
+      </c>
+      <c r="K79">
+        <v>531</v>
       </c>
     </row>
     <row r="80">
@@ -2706,28 +3183,34 @@
         <v>2026-04-20</v>
       </c>
       <c r="B80">
-        <v>5961749</v>
+        <v>10216535</v>
       </c>
       <c r="C80">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="D80">
-        <v>1</v>
+        <v>41934</v>
       </c>
       <c r="E80">
-        <v>79</v>
+        <v>1397230</v>
       </c>
       <c r="F80">
-        <v>8206</v>
+        <v>1439164</v>
       </c>
       <c r="G80">
-        <v>6.15</v>
+        <v>609.9</v>
       </c>
       <c r="H80">
-        <v>3028</v>
-      </c>
-      <c r="I80" t="str">
-        <v>facebook</v>
+        <v>2</v>
+      </c>
+      <c r="I80">
+        <v>10234</v>
+      </c>
+      <c r="J80">
+        <v>5.51</v>
+      </c>
+      <c r="K80">
+        <v>564</v>
       </c>
     </row>
     <row r="81">
@@ -2735,28 +3218,34 @@
         <v>2026-04-21</v>
       </c>
       <c r="B81">
-        <v>6749694</v>
+        <v>15826772</v>
       </c>
       <c r="C81">
-        <v>59</v>
+        <v>132</v>
       </c>
       <c r="D81">
+        <v>1822425</v>
+      </c>
+      <c r="E81">
+        <v>762199</v>
+      </c>
+      <c r="F81">
+        <v>2584624</v>
+      </c>
+      <c r="G81">
+        <v>512.3</v>
+      </c>
+      <c r="H81">
         <v>1</v>
       </c>
-      <c r="E81">
-        <v>80</v>
-      </c>
-      <c r="F81">
-        <v>6817</v>
-      </c>
-      <c r="G81">
-        <v>3.5</v>
-      </c>
-      <c r="H81">
-        <v>954</v>
-      </c>
-      <c r="I81" t="str">
-        <v>instagram</v>
+      <c r="I81">
+        <v>4863</v>
+      </c>
+      <c r="J81">
+        <v>3.28</v>
+      </c>
+      <c r="K81">
+        <v>160</v>
       </c>
     </row>
     <row r="82">
@@ -2764,28 +3253,34 @@
         <v>2026-04-22</v>
       </c>
       <c r="B82">
-        <v>6247640</v>
+        <v>16614173</v>
       </c>
       <c r="C82">
-        <v>57</v>
+        <v>138</v>
       </c>
       <c r="D82">
-        <v>1</v>
+        <v>890070</v>
       </c>
       <c r="E82">
-        <v>80</v>
+        <v>1875470</v>
       </c>
       <c r="F82">
-        <v>6165</v>
+        <v>2765540</v>
       </c>
       <c r="G82">
-        <v>7.57</v>
+        <v>500.8</v>
       </c>
       <c r="H82">
-        <v>1400</v>
-      </c>
-      <c r="I82" t="str">
-        <v>both</v>
+        <v>2</v>
+      </c>
+      <c r="I82">
+        <v>9460</v>
+      </c>
+      <c r="J82">
+        <v>5.19</v>
+      </c>
+      <c r="K82">
+        <v>491</v>
       </c>
     </row>
     <row r="83">
@@ -2793,28 +3288,34 @@
         <v>2026-04-23</v>
       </c>
       <c r="B83">
-        <v>6296630</v>
+        <v>17106299</v>
       </c>
       <c r="C83">
-        <v>58</v>
+        <v>143</v>
       </c>
       <c r="D83">
-        <v>1</v>
+        <v>2587572</v>
       </c>
       <c r="E83">
-        <v>81</v>
+        <v>293560</v>
       </c>
       <c r="F83">
-        <v>8758</v>
+        <v>2881132</v>
       </c>
       <c r="G83">
-        <v>4.61</v>
+        <v>493.7</v>
       </c>
       <c r="H83">
-        <v>2422</v>
-      </c>
-      <c r="I83" t="str">
-        <v>facebook</v>
+        <v>0</v>
+      </c>
+      <c r="I83">
+        <v>3992</v>
+      </c>
+      <c r="J83">
+        <v>2.91</v>
+      </c>
+      <c r="K83">
+        <v>116</v>
       </c>
     </row>
     <row r="84">
@@ -2822,28 +3323,34 @@
         <v>2026-04-24</v>
       </c>
       <c r="B84">
-        <v>6880279</v>
+        <v>16122047</v>
       </c>
       <c r="C84">
-        <v>61</v>
+        <v>134</v>
       </c>
       <c r="D84">
-        <v>1</v>
+        <v>1006493</v>
       </c>
       <c r="E84">
-        <v>81</v>
+        <v>1645393</v>
       </c>
       <c r="F84">
-        <v>9281</v>
+        <v>2651886</v>
       </c>
       <c r="G84">
-        <v>6.81</v>
+        <v>507.9</v>
       </c>
       <c r="H84">
-        <v>3792</v>
-      </c>
-      <c r="I84" t="str">
-        <v>instagram</v>
+        <v>2</v>
+      </c>
+      <c r="I84">
+        <v>7911</v>
+      </c>
+      <c r="J84">
+        <v>4.55</v>
+      </c>
+      <c r="K84">
+        <v>360</v>
       </c>
     </row>
     <row r="85">
@@ -2851,28 +3358,34 @@
         <v>2026-04-25</v>
       </c>
       <c r="B85">
-        <v>5158422</v>
+        <v>18385827</v>
       </c>
       <c r="C85">
-        <v>51</v>
+        <v>153</v>
       </c>
       <c r="D85">
-        <v>0</v>
+        <v>651974</v>
       </c>
       <c r="E85">
-        <v>0</v>
+        <v>2538763</v>
       </c>
       <c r="F85">
-        <v>101</v>
+        <v>3190737</v>
       </c>
       <c r="G85">
-        <v>0.98</v>
+        <v>476.2</v>
       </c>
       <c r="H85">
-        <v>11</v>
-      </c>
-      <c r="I85" t="str">
-        <v/>
+        <v>2</v>
+      </c>
+      <c r="I85">
+        <v>13766</v>
+      </c>
+      <c r="J85">
+        <v>6.99</v>
+      </c>
+      <c r="K85">
+        <v>962</v>
       </c>
     </row>
     <row r="86">
@@ -2880,28 +3393,34 @@
         <v>2026-04-26</v>
       </c>
       <c r="B86">
-        <v>5758471</v>
+        <v>26358268</v>
       </c>
       <c r="C86">
-        <v>60</v>
+        <v>220</v>
       </c>
       <c r="D86">
-        <v>0</v>
+        <v>2454672</v>
       </c>
       <c r="E86">
-        <v>0</v>
+        <v>2960188</v>
       </c>
       <c r="F86">
-        <v>296</v>
+        <v>5414860</v>
       </c>
       <c r="G86">
-        <v>1.97</v>
+        <v>386.8</v>
       </c>
       <c r="H86">
-        <v>4</v>
-      </c>
-      <c r="I86" t="str">
-        <v/>
+        <v>2</v>
+      </c>
+      <c r="I86">
+        <v>13403</v>
+      </c>
+      <c r="J86">
+        <v>6.83</v>
+      </c>
+      <c r="K86">
+        <v>915</v>
       </c>
     </row>
     <row r="87">
@@ -2909,28 +3428,34 @@
         <v>2026-04-27</v>
       </c>
       <c r="B87">
-        <v>7566959</v>
+        <v>19960630</v>
       </c>
       <c r="C87">
-        <v>78</v>
+        <v>166</v>
       </c>
       <c r="D87">
-        <v>1</v>
+        <v>2273525</v>
       </c>
       <c r="E87">
-        <v>83</v>
+        <v>1316245</v>
       </c>
       <c r="F87">
-        <v>9743</v>
+        <v>3589770</v>
       </c>
       <c r="G87">
-        <v>6.27</v>
+        <v>456</v>
       </c>
       <c r="H87">
-        <v>3665</v>
-      </c>
-      <c r="I87" t="str">
-        <v>facebook</v>
+        <v>2</v>
+      </c>
+      <c r="I87">
+        <v>7452</v>
+      </c>
+      <c r="J87">
+        <v>4.35</v>
+      </c>
+      <c r="K87">
+        <v>324</v>
       </c>
     </row>
     <row r="88">
@@ -2938,28 +3463,34 @@
         <v>2026-04-28</v>
       </c>
       <c r="B88">
-        <v>6711448</v>
+        <v>16811024</v>
       </c>
       <c r="C88">
-        <v>68</v>
+        <v>140</v>
       </c>
       <c r="D88">
-        <v>1</v>
+        <v>886383</v>
       </c>
       <c r="E88">
-        <v>83</v>
+        <v>1925161</v>
       </c>
       <c r="F88">
-        <v>5879</v>
+        <v>2811544</v>
       </c>
       <c r="G88">
-        <v>5.61</v>
+        <v>497.9</v>
       </c>
       <c r="H88">
-        <v>989</v>
-      </c>
-      <c r="I88" t="str">
-        <v>instagram</v>
+        <v>2</v>
+      </c>
+      <c r="I88">
+        <v>9653</v>
+      </c>
+      <c r="J88">
+        <v>5.27</v>
+      </c>
+      <c r="K88">
+        <v>509</v>
       </c>
     </row>
     <row r="89">
@@ -2967,28 +3498,34 @@
         <v>2026-04-29</v>
       </c>
       <c r="B89">
-        <v>7187445</v>
+        <v>20748031</v>
       </c>
       <c r="C89">
-        <v>73</v>
+        <v>173</v>
       </c>
       <c r="D89">
-        <v>1</v>
+        <v>1187409</v>
       </c>
       <c r="E89">
-        <v>84</v>
+        <v>2609317</v>
       </c>
       <c r="F89">
-        <v>8346</v>
+        <v>3796726</v>
       </c>
       <c r="G89">
-        <v>3.99</v>
+        <v>446.5</v>
       </c>
       <c r="H89">
-        <v>1332</v>
-      </c>
-      <c r="I89" t="str">
-        <v>both</v>
+        <v>2</v>
+      </c>
+      <c r="I89">
+        <v>12823</v>
+      </c>
+      <c r="J89">
+        <v>6.59</v>
+      </c>
+      <c r="K89">
+        <v>845</v>
       </c>
     </row>
     <row r="90">
@@ -2996,28 +3533,34 @@
         <v>2026-04-30</v>
       </c>
       <c r="B90">
-        <v>6570393</v>
+        <v>17696850</v>
       </c>
       <c r="C90">
-        <v>58</v>
+        <v>147</v>
       </c>
       <c r="D90">
-        <v>1</v>
+        <v>1101983</v>
       </c>
       <c r="E90">
-        <v>84</v>
+        <v>1920416</v>
       </c>
       <c r="F90">
-        <v>5180</v>
+        <v>3022399</v>
       </c>
       <c r="G90">
-        <v>3.55</v>
+        <v>485.5</v>
       </c>
       <c r="H90">
-        <v>736</v>
-      </c>
-      <c r="I90" t="str">
-        <v>facebook</v>
+        <v>2</v>
+      </c>
+      <c r="I90">
+        <v>9169</v>
+      </c>
+      <c r="J90">
+        <v>5.07</v>
+      </c>
+      <c r="K90">
+        <v>465</v>
       </c>
     </row>
     <row r="91">
@@ -3025,33 +3568,153 @@
         <v>2026-05-01</v>
       </c>
       <c r="B91">
-        <v>6103819</v>
+        <v>21437008</v>
       </c>
       <c r="C91">
-        <v>57</v>
+        <v>179</v>
       </c>
       <c r="D91">
-        <v>1</v>
+        <v>1104957</v>
       </c>
       <c r="E91">
-        <v>85</v>
+        <v>2876925</v>
       </c>
       <c r="F91">
-        <v>8041</v>
+        <v>3981882</v>
       </c>
       <c r="G91">
-        <v>6.71</v>
+        <v>438.4</v>
       </c>
       <c r="H91">
-        <v>3237</v>
-      </c>
-      <c r="I91" t="str">
-        <v>instagram</v>
+        <v>2</v>
+      </c>
+      <c r="I91">
+        <v>14565</v>
+      </c>
+      <c r="J91">
+        <v>7.32</v>
+      </c>
+      <c r="K91">
+        <v>1066</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I91"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K91"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B15"/>
+  <cols>
+    <col min="1" max="1" width="25.83203125" customWidth="1"/>
+    <col min="2" max="2" width="60.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Thông tin Dataset</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Nguồn gốc data</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Real "Advertising Spend vs Sales" dataset</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>URL nguồn</v>
+      </c>
+      <c r="B4" t="str">
+        <v>https://github.com/prasertcbs/basic-dataset/blob/master/marketing.csv</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Mô tả gốc</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Dữ liệu thật về chi phí quảng cáo YouTube/Facebook/Báo vs Doanh số</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Số quan sát</v>
+      </c>
+      <c r="B6" t="str">
+        <v>200 observations (dùng 90 ngày đầu)</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Transform áp dụng</v>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>- Thêm ngày</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Bắt đầu từ 01/02/2026, mỗi row = 1 ngày</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>- Đơn vị tiền</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Quy đổi sang VND (spend × 500,000 | doanh thu × 2,000,000)</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>- Ngành</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Sản phẩm skincare / mỹ phẩm Việt Nam</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Hướng dẫn dùng</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Upload file này → AI sẽ phân tích mối quan hệ chi phí QC vs doanh thu</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Bạn có thể thay bằng file Excel của doanh nghiệp mình với bất kỳ cột nào</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add ML-driven campaign analytics and BI dashboard
</commit_message>
<xml_diff>
--- a/backend/data/sample-campaign-skincare.xlsx
+++ b/backend/data/sample-campaign-skincare.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K91"/>
+  <dimension ref="A1:L91"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -406,11 +406,12 @@
     <col min="4" max="4" width="24.83203125" customWidth="1"/>
     <col min="5" max="5" width="26.83203125" customWidth="1"/>
     <col min="6" max="6" width="22.83203125" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="22.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="22.83203125" customWidth="1"/>
+    <col min="8" max="8" width="10.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" customWidth="1"/>
+    <col min="11" max="11" width="22.83203125" customWidth="1"/>
+    <col min="12" max="12" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -430,21 +431,24 @@
         <v>Chi phí QC Facebook (VND)</v>
       </c>
       <c r="F1" t="str">
+        <v>Chi phí QC Báo (VND)</v>
+      </c>
+      <c r="G1" t="str">
         <v>Tổng chi phí QC (VND)</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>ROI (%)</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Số bài đăng</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Lượt tiếp cận</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>Tỷ lệ tương tác (%)</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Lượt click</v>
       </c>
     </row>
@@ -453,34 +457,37 @@
         <v>2026-02-01</v>
       </c>
       <c r="B2">
-        <v>26751969</v>
+        <v>53040000</v>
       </c>
       <c r="C2">
-        <v>223</v>
+        <v>442</v>
       </c>
       <c r="D2">
-        <v>2789619</v>
+        <v>138060000</v>
       </c>
       <c r="E2">
-        <v>2748249</v>
+        <v>22680000</v>
       </c>
       <c r="F2">
-        <v>5537868</v>
+        <v>41520000</v>
       </c>
       <c r="G2">
-        <v>383.1</v>
+        <v>202260000</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>-73.8</v>
       </c>
       <c r="I2">
-        <v>12145</v>
+        <v>2</v>
       </c>
       <c r="J2">
-        <v>6.31</v>
+        <v>12182</v>
       </c>
       <c r="K2">
-        <v>766</v>
+        <v>6.33</v>
+      </c>
+      <c r="L2">
+        <v>771</v>
       </c>
     </row>
     <row r="3">
@@ -488,34 +495,37 @@
         <v>2026-02-02</v>
       </c>
       <c r="B3">
-        <v>15236220</v>
+        <v>24960000</v>
       </c>
       <c r="C3">
-        <v>127</v>
+        <v>208</v>
       </c>
       <c r="D3">
-        <v>389631</v>
+        <v>26700000</v>
       </c>
       <c r="E3">
-        <v>2062561</v>
+        <v>23580000</v>
       </c>
       <c r="F3">
-        <v>2452192</v>
+        <v>27060000</v>
       </c>
       <c r="G3">
-        <v>521.3</v>
+        <v>77340000</v>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>-67.7</v>
       </c>
       <c r="I3">
-        <v>12508</v>
+        <v>2</v>
       </c>
       <c r="J3">
-        <v>6.46</v>
+        <v>12547</v>
       </c>
       <c r="K3">
-        <v>808</v>
+        <v>6.48</v>
+      </c>
+      <c r="L3">
+        <v>813</v>
       </c>
     </row>
     <row r="4">
@@ -523,34 +533,37 @@
         <v>2026-02-03</v>
       </c>
       <c r="B4">
-        <v>14153543</v>
+        <v>22320000</v>
       </c>
       <c r="C4">
-        <v>118</v>
+        <v>186</v>
       </c>
       <c r="D4">
-        <v>130644</v>
+        <v>10320000</v>
       </c>
       <c r="E4">
-        <v>2086001</v>
+        <v>27060000</v>
       </c>
       <c r="F4">
-        <v>2216645</v>
+        <v>41640000</v>
       </c>
       <c r="G4">
-        <v>538.5</v>
+        <v>79020000</v>
       </c>
       <c r="H4">
-        <v>2</v>
+        <v>-71.8</v>
       </c>
       <c r="I4">
-        <v>14105</v>
+        <v>2</v>
       </c>
       <c r="J4">
-        <v>7.13</v>
+        <v>13955</v>
       </c>
       <c r="K4">
-        <v>1006</v>
+        <v>7.06</v>
+      </c>
+      <c r="L4">
+        <v>985</v>
       </c>
     </row>
     <row r="5">
@@ -558,34 +571,37 @@
         <v>2026-02-04</v>
       </c>
       <c r="B5">
-        <v>23208661</v>
+        <v>44160000</v>
       </c>
       <c r="C5">
-        <v>193</v>
+        <v>368</v>
       </c>
       <c r="D5">
-        <v>1699722</v>
+        <v>90720000</v>
       </c>
       <c r="E5">
-        <v>2775712</v>
+        <v>24540000</v>
       </c>
       <c r="F5">
-        <v>4475434</v>
+        <v>35040000</v>
       </c>
       <c r="G5">
-        <v>418.6</v>
+        <v>150300000</v>
       </c>
       <c r="H5">
-        <v>2</v>
+        <v>-70.6</v>
       </c>
       <c r="I5">
-        <v>12992</v>
+        <v>2</v>
       </c>
       <c r="J5">
-        <v>6.66</v>
+        <v>12935</v>
       </c>
       <c r="K5">
-        <v>865</v>
+        <v>6.64</v>
+      </c>
+      <c r="L5">
+        <v>859</v>
       </c>
     </row>
     <row r="6">
@@ -593,33 +609,36 @@
         <v>2026-02-05</v>
       </c>
       <c r="B6">
-        <v>17696850</v>
+        <v>30960000</v>
       </c>
       <c r="C6">
-        <v>147</v>
+        <v>258</v>
       </c>
       <c r="D6">
-        <v>2206407</v>
+        <v>108540000</v>
       </c>
       <c r="E6">
-        <v>815992</v>
+        <v>6480000</v>
       </c>
       <c r="F6">
-        <v>3022399</v>
+        <v>35040000</v>
       </c>
       <c r="G6">
-        <v>485.5</v>
+        <v>150060000</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>-79.4</v>
       </c>
       <c r="I6">
-        <v>5613</v>
+        <v>2</v>
       </c>
       <c r="J6">
+        <v>5623</v>
+      </c>
+      <c r="K6">
         <v>3.59</v>
       </c>
-      <c r="K6">
+      <c r="L6">
         <v>202</v>
       </c>
     </row>
@@ -628,34 +647,37 @@
         <v>2026-02-06</v>
       </c>
       <c r="B7">
-        <v>12086614</v>
+        <v>17280000</v>
       </c>
       <c r="C7">
-        <v>101</v>
+        <v>144</v>
       </c>
       <c r="D7">
-        <v>51809</v>
+        <v>5220000</v>
       </c>
       <c r="E7">
-        <v>1741197</v>
+        <v>29400000</v>
       </c>
       <c r="F7">
-        <v>1793006</v>
+        <v>45000000</v>
       </c>
       <c r="G7">
-        <v>574.1</v>
+        <v>79620000</v>
       </c>
       <c r="H7">
-        <v>2</v>
+        <v>-78.3</v>
       </c>
       <c r="I7">
-        <v>14831</v>
+        <v>2</v>
       </c>
       <c r="J7">
-        <v>7.43</v>
+        <v>14903</v>
       </c>
       <c r="K7">
-        <v>1102</v>
+        <v>7.46</v>
+      </c>
+      <c r="L7">
+        <v>1112</v>
       </c>
     </row>
     <row r="8">
@@ -663,34 +685,37 @@
         <v>2026-02-07</v>
       </c>
       <c r="B8">
-        <v>16614173</v>
+        <v>27600000</v>
       </c>
       <c r="C8">
-        <v>138</v>
+        <v>230</v>
       </c>
       <c r="D8">
-        <v>624604</v>
+        <v>34560000</v>
       </c>
       <c r="E8">
-        <v>2140936</v>
+        <v>19260000</v>
       </c>
       <c r="F8">
-        <v>2765540</v>
+        <v>13800000</v>
       </c>
       <c r="G8">
-        <v>500.8</v>
+        <v>67620000</v>
       </c>
       <c r="H8">
-        <v>2</v>
+        <v>-59.2</v>
       </c>
       <c r="I8">
-        <v>10935</v>
+        <v>2</v>
       </c>
       <c r="J8">
-        <v>5.81</v>
+        <v>10798</v>
       </c>
       <c r="K8">
-        <v>635</v>
+        <v>5.75</v>
+      </c>
+      <c r="L8">
+        <v>621</v>
       </c>
     </row>
     <row r="9">
@@ -698,34 +723,37 @@
         <v>2026-02-08</v>
       </c>
       <c r="B9">
-        <v>17992126</v>
+        <v>31680000</v>
       </c>
       <c r="C9">
-        <v>150</v>
+        <v>264</v>
       </c>
       <c r="D9">
-        <v>1555091</v>
+        <v>72120000</v>
       </c>
       <c r="E9">
-        <v>1538988</v>
+        <v>11520000</v>
       </c>
       <c r="F9">
-        <v>3094079</v>
+        <v>6960000</v>
       </c>
       <c r="G9">
-        <v>481.5</v>
+        <v>90600000</v>
       </c>
       <c r="H9">
-        <v>2</v>
+        <v>-65</v>
       </c>
       <c r="I9">
-        <v>7742</v>
+        <v>2</v>
       </c>
       <c r="J9">
-        <v>4.48</v>
+        <v>7664</v>
       </c>
       <c r="K9">
-        <v>347</v>
+        <v>4.44</v>
+      </c>
+      <c r="L9">
+        <v>340</v>
       </c>
     </row>
     <row r="10">
@@ -733,33 +761,36 @@
         <v>2026-02-09</v>
       </c>
       <c r="B10">
-        <v>9724409</v>
+        <v>11520000</v>
       </c>
       <c r="C10">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="D10">
-        <v>484673</v>
+        <v>5160000</v>
       </c>
       <c r="E10">
-        <v>866024</v>
+        <v>1260000</v>
       </c>
       <c r="F10">
-        <v>1350697</v>
+        <v>600000</v>
       </c>
       <c r="G10">
-        <v>620</v>
+        <v>7020000</v>
       </c>
       <c r="H10">
-        <v>2</v>
+        <v>64.1</v>
       </c>
       <c r="I10">
-        <v>3508</v>
+        <v>2</v>
       </c>
       <c r="J10">
+        <v>3510</v>
+      </c>
+      <c r="K10">
         <v>2.71</v>
       </c>
-      <c r="K10">
+      <c r="L10">
         <v>95</v>
       </c>
     </row>
@@ -768,33 +799,36 @@
         <v>2026-02-10</v>
       </c>
       <c r="B11">
-        <v>15433071</v>
+        <v>25440000</v>
       </c>
       <c r="C11">
-        <v>129</v>
+        <v>212</v>
       </c>
       <c r="D11">
-        <v>2286317</v>
+        <v>119520000</v>
       </c>
       <c r="E11">
-        <v>209709</v>
+        <v>1560000</v>
       </c>
       <c r="F11">
-        <v>2496026</v>
+        <v>12720000</v>
       </c>
       <c r="G11">
-        <v>518.3</v>
+        <v>133800000</v>
       </c>
       <c r="H11">
-        <v>0</v>
+        <v>-81</v>
       </c>
       <c r="I11">
-        <v>3629</v>
+        <v>2</v>
       </c>
       <c r="J11">
+        <v>3632</v>
+      </c>
+      <c r="K11">
         <v>2.76</v>
       </c>
-      <c r="K11">
+      <c r="L11">
         <v>100</v>
       </c>
     </row>
@@ -803,33 +837,36 @@
         <v>2026-02-11</v>
       </c>
       <c r="B12">
-        <v>13464567</v>
+        <v>20640000</v>
       </c>
       <c r="C12">
-        <v>112</v>
+        <v>172</v>
       </c>
       <c r="D12">
-        <v>1324730</v>
+        <v>39720000</v>
       </c>
       <c r="E12">
-        <v>746905</v>
+        <v>3480000</v>
       </c>
       <c r="F12">
-        <v>2071635</v>
+        <v>14520000</v>
       </c>
       <c r="G12">
-        <v>549.9</v>
+        <v>57720000</v>
       </c>
       <c r="H12">
-        <v>2</v>
+        <v>-64.2</v>
       </c>
       <c r="I12">
-        <v>4403</v>
+        <v>2</v>
       </c>
       <c r="J12">
-        <v>3.08</v>
+        <v>4409</v>
       </c>
       <c r="K12">
+        <v>3.09</v>
+      </c>
+      <c r="L12">
         <v>136</v>
       </c>
     </row>
@@ -838,34 +875,37 @@
         <v>2026-02-12</v>
       </c>
       <c r="B13">
-        <v>22125984</v>
+        <v>41760000</v>
       </c>
       <c r="C13">
-        <v>184</v>
+        <v>348</v>
       </c>
       <c r="D13">
-        <v>2489511</v>
+        <v>128700000</v>
       </c>
       <c r="E13">
-        <v>1681324</v>
+        <v>14400000</v>
       </c>
       <c r="F13">
-        <v>4170835</v>
+        <v>2400000</v>
       </c>
       <c r="G13">
-        <v>430.5</v>
+        <v>145500000</v>
       </c>
       <c r="H13">
-        <v>2</v>
+        <v>-71.3</v>
       </c>
       <c r="I13">
-        <v>8806</v>
+        <v>2</v>
       </c>
       <c r="J13">
-        <v>4.92</v>
+        <v>8830</v>
       </c>
       <c r="K13">
-        <v>433</v>
+        <v>4.93</v>
+      </c>
+      <c r="L13">
+        <v>435</v>
       </c>
     </row>
     <row r="14">
@@ -873,34 +913,37 @@
         <v>2026-02-13</v>
       </c>
       <c r="B14">
-        <v>14055118</v>
+        <v>22560000</v>
       </c>
       <c r="C14">
-        <v>117</v>
+        <v>188</v>
       </c>
       <c r="D14">
-        <v>222842</v>
+        <v>14220000</v>
       </c>
       <c r="E14">
-        <v>1972855</v>
+        <v>21060000</v>
       </c>
       <c r="F14">
-        <v>2195697</v>
+        <v>39060000</v>
       </c>
       <c r="G14">
-        <v>540.1</v>
+        <v>74340000</v>
       </c>
       <c r="H14">
-        <v>2</v>
+        <v>-69.7</v>
       </c>
       <c r="I14">
-        <v>11492</v>
+        <v>2</v>
       </c>
       <c r="J14">
-        <v>6.04</v>
+        <v>11526</v>
       </c>
       <c r="K14">
-        <v>694</v>
+        <v>6.05</v>
+      </c>
+      <c r="L14">
+        <v>697</v>
       </c>
     </row>
     <row r="15">
@@ -908,34 +951,37 @@
         <v>2026-02-14</v>
       </c>
       <c r="B15">
-        <v>14547244</v>
+        <v>23280000</v>
       </c>
       <c r="C15">
-        <v>121</v>
+        <v>194</v>
       </c>
       <c r="D15">
-        <v>1542866</v>
+        <v>58440000</v>
       </c>
       <c r="E15">
-        <v>758348</v>
+        <v>4440000</v>
       </c>
       <c r="F15">
-        <v>2301214</v>
+        <v>4320000</v>
       </c>
       <c r="G15">
-        <v>532.2</v>
+        <v>67200000</v>
       </c>
       <c r="H15">
-        <v>2</v>
+        <v>-65.4</v>
       </c>
       <c r="I15">
-        <v>4839</v>
+        <v>2</v>
       </c>
       <c r="J15">
-        <v>3.27</v>
+        <v>4798</v>
       </c>
       <c r="K15">
-        <v>158</v>
+        <v>3.25</v>
+      </c>
+      <c r="L15">
+        <v>156</v>
       </c>
     </row>
     <row r="16">
@@ -943,34 +989,37 @@
         <v>2026-02-15</v>
       </c>
       <c r="B16">
-        <v>23700787</v>
+        <v>45600000</v>
       </c>
       <c r="C16">
-        <v>198</v>
+        <v>380</v>
       </c>
       <c r="D16">
-        <v>2345365</v>
+        <v>122640000</v>
       </c>
       <c r="E16">
-        <v>2271623</v>
+        <v>19200000</v>
       </c>
       <c r="F16">
-        <v>4616988</v>
+        <v>27600000</v>
       </c>
       <c r="G16">
-        <v>413.3</v>
+        <v>169440000</v>
       </c>
       <c r="H16">
-        <v>2</v>
+        <v>-73.1</v>
       </c>
       <c r="I16">
-        <v>10960</v>
+        <v>2</v>
       </c>
       <c r="J16">
-        <v>5.82</v>
+        <v>10773</v>
       </c>
       <c r="K16">
-        <v>638</v>
+        <v>5.74</v>
+      </c>
+      <c r="L16">
+        <v>618</v>
       </c>
     </row>
     <row r="17">
@@ -978,34 +1027,37 @@
         <v>2026-02-16</v>
       </c>
       <c r="B17">
-        <v>27047244</v>
+        <v>53760000</v>
       </c>
       <c r="C17">
-        <v>225</v>
+        <v>448</v>
       </c>
       <c r="D17">
-        <v>2288974</v>
+        <v>117000000</v>
       </c>
       <c r="E17">
-        <v>3341964</v>
+        <v>28320000</v>
       </c>
       <c r="F17">
-        <v>5630938</v>
+        <v>31380000</v>
       </c>
       <c r="G17">
-        <v>380.3</v>
+        <v>176700000</v>
       </c>
       <c r="H17">
-        <v>2</v>
+        <v>-69.6</v>
       </c>
       <c r="I17">
-        <v>14540</v>
+        <v>2</v>
       </c>
       <c r="J17">
-        <v>7.31</v>
+        <v>14466</v>
       </c>
       <c r="K17">
-        <v>1063</v>
+        <v>7.28</v>
+      </c>
+      <c r="L17">
+        <v>1053</v>
       </c>
     </row>
     <row r="18">
@@ -1013,34 +1065,37 @@
         <v>2026-02-17</v>
       </c>
       <c r="B18">
-        <v>17303150</v>
+        <v>30000000</v>
       </c>
       <c r="C18">
-        <v>144</v>
+        <v>250</v>
       </c>
       <c r="D18">
-        <v>690756</v>
+        <v>40320000</v>
       </c>
       <c r="E18">
-        <v>2237155</v>
+        <v>21960000</v>
       </c>
       <c r="F18">
-        <v>2927911</v>
+        <v>68700000</v>
       </c>
       <c r="G18">
-        <v>491</v>
+        <v>130980000</v>
       </c>
       <c r="H18">
-        <v>2</v>
+        <v>-77.1</v>
       </c>
       <c r="I18">
-        <v>11855</v>
+        <v>2</v>
       </c>
       <c r="J18">
-        <v>6.19</v>
+        <v>11891</v>
       </c>
       <c r="K18">
-        <v>734</v>
+        <v>6.2</v>
+      </c>
+      <c r="L18">
+        <v>737</v>
       </c>
     </row>
     <row r="19">
@@ -1048,34 +1103,37 @@
         <v>2026-02-18</v>
       </c>
       <c r="B19">
-        <v>29015748</v>
+        <v>58320000</v>
       </c>
       <c r="C19">
-        <v>242</v>
+        <v>486</v>
       </c>
       <c r="D19">
-        <v>3400842</v>
+        <v>168780000</v>
       </c>
       <c r="E19">
-        <v>2868387</v>
+        <v>23400000</v>
       </c>
       <c r="F19">
-        <v>6269229</v>
+        <v>33000000</v>
       </c>
       <c r="G19">
-        <v>362.8</v>
+        <v>225180000</v>
       </c>
       <c r="H19">
-        <v>2</v>
+        <v>-74.1</v>
       </c>
       <c r="I19">
-        <v>12581</v>
+        <v>2</v>
       </c>
       <c r="J19">
-        <v>6.49</v>
+        <v>12474</v>
       </c>
       <c r="K19">
-        <v>817</v>
+        <v>6.45</v>
+      </c>
+      <c r="L19">
+        <v>805</v>
       </c>
     </row>
     <row r="20">
@@ -1083,34 +1141,37 @@
         <v>2026-02-19</v>
       </c>
       <c r="B20">
-        <v>16122047</v>
+        <v>27360000</v>
       </c>
       <c r="C20">
-        <v>134</v>
+        <v>228</v>
       </c>
       <c r="D20">
-        <v>948459</v>
+        <v>41640000</v>
       </c>
       <c r="E20">
-        <v>1703427</v>
+        <v>12000000</v>
       </c>
       <c r="F20">
-        <v>2651886</v>
+        <v>11040000</v>
       </c>
       <c r="G20">
-        <v>507.9</v>
+        <v>64680000</v>
       </c>
       <c r="H20">
-        <v>2</v>
+        <v>-57.7</v>
       </c>
       <c r="I20">
-        <v>7960</v>
+        <v>2</v>
       </c>
       <c r="J20">
-        <v>4.57</v>
+        <v>7858</v>
       </c>
       <c r="K20">
-        <v>364</v>
+        <v>4.52</v>
+      </c>
+      <c r="L20">
+        <v>355</v>
       </c>
     </row>
     <row r="21">
@@ -1118,34 +1179,37 @@
         <v>2026-02-20</v>
       </c>
       <c r="B21">
-        <v>19370079</v>
+        <v>34560000</v>
       </c>
       <c r="C21">
-        <v>161</v>
+        <v>288</v>
       </c>
       <c r="D21">
-        <v>1735942</v>
+        <v>88800000</v>
       </c>
       <c r="E21">
-        <v>1701866</v>
+        <v>13740000</v>
       </c>
       <c r="F21">
-        <v>3437808</v>
+        <v>10980000</v>
       </c>
       <c r="G21">
-        <v>463.4</v>
+        <v>113520000</v>
       </c>
       <c r="H21">
-        <v>2</v>
+        <v>-69.6</v>
       </c>
       <c r="I21">
-        <v>8782</v>
+        <v>2</v>
       </c>
       <c r="J21">
-        <v>4.91</v>
+        <v>8563</v>
       </c>
       <c r="K21">
-        <v>431</v>
+        <v>4.82</v>
+      </c>
+      <c r="L21">
+        <v>413</v>
       </c>
     </row>
     <row r="22">
@@ -1153,34 +1217,37 @@
         <v>2026-02-21</v>
       </c>
       <c r="B22">
-        <v>22716535</v>
+        <v>43200000</v>
       </c>
       <c r="C22">
-        <v>189</v>
+        <v>360</v>
       </c>
       <c r="D22">
-        <v>2457662</v>
+        <v>131400000</v>
       </c>
       <c r="E22">
-        <v>1878155</v>
+        <v>16320000</v>
       </c>
       <c r="F22">
-        <v>4335817</v>
+        <v>31800000</v>
       </c>
       <c r="G22">
-        <v>423.9</v>
+        <v>179520000</v>
       </c>
       <c r="H22">
-        <v>2</v>
+        <v>-75.9</v>
       </c>
       <c r="I22">
-        <v>9702</v>
+        <v>2</v>
       </c>
       <c r="J22">
-        <v>5.29</v>
+        <v>9607</v>
       </c>
       <c r="K22">
-        <v>513</v>
+        <v>5.25</v>
+      </c>
+      <c r="L22">
+        <v>504</v>
       </c>
     </row>
     <row r="23">
@@ -1188,34 +1255,37 @@
         <v>2026-02-22</v>
       </c>
       <c r="B23">
-        <v>17303150</v>
+        <v>31200000</v>
       </c>
       <c r="C23">
-        <v>144</v>
+        <v>260</v>
       </c>
       <c r="D23">
-        <v>2569400</v>
+        <v>142740000</v>
       </c>
       <c r="E23">
-        <v>358511</v>
+        <v>3120000</v>
       </c>
       <c r="F23">
-        <v>2927911</v>
+        <v>14040000</v>
       </c>
       <c r="G23">
-        <v>491</v>
+        <v>159900000</v>
       </c>
       <c r="H23">
-        <v>1</v>
+        <v>-80.5</v>
       </c>
       <c r="I23">
-        <v>4234</v>
+        <v>2</v>
       </c>
       <c r="J23">
-        <v>3.01</v>
+        <v>4263</v>
       </c>
       <c r="K23">
-        <v>127</v>
+        <v>3.03</v>
+      </c>
+      <c r="L23">
+        <v>129</v>
       </c>
     </row>
     <row r="24">
@@ -1223,34 +1293,37 @@
         <v>2026-02-23</v>
       </c>
       <c r="B24">
-        <v>10511811</v>
+        <v>13440000</v>
       </c>
       <c r="C24">
-        <v>88</v>
+        <v>112</v>
       </c>
       <c r="D24">
-        <v>178769</v>
+        <v>7920000</v>
       </c>
       <c r="E24">
-        <v>1314405</v>
+        <v>9480000</v>
       </c>
       <c r="F24">
-        <v>1493174</v>
+        <v>29820000</v>
       </c>
       <c r="G24">
-        <v>604</v>
+        <v>47220000</v>
       </c>
       <c r="H24">
-        <v>2</v>
+        <v>-71.5</v>
       </c>
       <c r="I24">
-        <v>6847</v>
+        <v>2</v>
       </c>
       <c r="J24">
+        <v>6838</v>
+      </c>
+      <c r="K24">
         <v>4.1</v>
       </c>
-      <c r="K24">
-        <v>281</v>
+      <c r="L24">
+        <v>280</v>
       </c>
     </row>
     <row r="25">
@@ -1258,34 +1331,37 @@
         <v>2026-02-24</v>
       </c>
       <c r="B25">
-        <v>20255906</v>
+        <v>37200000</v>
       </c>
       <c r="C25">
-        <v>169</v>
+        <v>310</v>
       </c>
       <c r="D25">
-        <v>2527008</v>
+        <v>137100000</v>
       </c>
       <c r="E25">
-        <v>1139789</v>
+        <v>9960000</v>
       </c>
       <c r="F25">
-        <v>3666797</v>
+        <v>15540000</v>
       </c>
       <c r="G25">
-        <v>452.4</v>
+        <v>162600000</v>
       </c>
       <c r="H25">
-        <v>2</v>
+        <v>-77.1</v>
       </c>
       <c r="I25">
-        <v>7089</v>
+        <v>2</v>
       </c>
       <c r="J25">
-        <v>4.2</v>
+        <v>7032</v>
       </c>
       <c r="K25">
-        <v>298</v>
+        <v>4.18</v>
+      </c>
+      <c r="L25">
+        <v>294</v>
       </c>
     </row>
     <row r="26">
@@ -1293,34 +1369,37 @@
         <v>2026-02-25</v>
       </c>
       <c r="B26">
-        <v>14547244</v>
+        <v>23280000</v>
       </c>
       <c r="C26">
-        <v>121</v>
+        <v>194</v>
       </c>
       <c r="D26">
-        <v>1025359</v>
+        <v>37680000</v>
       </c>
       <c r="E26">
-        <v>1275855</v>
+        <v>7560000</v>
       </c>
       <c r="F26">
-        <v>2301214</v>
+        <v>11340000</v>
       </c>
       <c r="G26">
-        <v>532.2</v>
+        <v>56580000</v>
       </c>
       <c r="H26">
-        <v>2</v>
+        <v>-58.9</v>
       </c>
       <c r="I26">
-        <v>6048</v>
+        <v>2</v>
       </c>
       <c r="J26">
-        <v>3.77</v>
+        <v>6061</v>
       </c>
       <c r="K26">
-        <v>228</v>
+        <v>3.78</v>
+      </c>
+      <c r="L26">
+        <v>229</v>
       </c>
     </row>
     <row r="27">
@@ -1328,34 +1407,37 @@
         <v>2026-02-26</v>
       </c>
       <c r="B27">
-        <v>16811024</v>
+        <v>28800000</v>
       </c>
       <c r="C27">
-        <v>140</v>
+        <v>240</v>
       </c>
       <c r="D27">
-        <v>2579463</v>
+        <v>157500000</v>
       </c>
       <c r="E27">
-        <v>232081</v>
+        <v>2040000</v>
       </c>
       <c r="F27">
-        <v>2811544</v>
+        <v>11760000</v>
       </c>
       <c r="G27">
-        <v>497.9</v>
+        <v>171300000</v>
       </c>
       <c r="H27">
-        <v>0</v>
+        <v>-83.2</v>
       </c>
       <c r="I27">
-        <v>3847</v>
+        <v>2</v>
       </c>
       <c r="J27">
-        <v>2.85</v>
+        <v>3826</v>
       </c>
       <c r="K27">
-        <v>110</v>
+        <v>2.84</v>
+      </c>
+      <c r="L27">
+        <v>109</v>
       </c>
     </row>
     <row r="28">
@@ -1363,34 +1445,37 @@
         <v>2026-02-27</v>
       </c>
       <c r="B28">
-        <v>19763780</v>
+        <v>36000000</v>
       </c>
       <c r="C28">
-        <v>165</v>
+        <v>300</v>
       </c>
       <c r="D28">
-        <v>1583896</v>
+        <v>85500000</v>
       </c>
       <c r="E28">
-        <v>1954910</v>
+        <v>17400000</v>
       </c>
       <c r="F28">
-        <v>3538806</v>
+        <v>7320000</v>
       </c>
       <c r="G28">
-        <v>458.5</v>
+        <v>110220000</v>
       </c>
       <c r="H28">
-        <v>2</v>
+        <v>-67.3</v>
       </c>
       <c r="I28">
-        <v>10089</v>
+        <v>2</v>
       </c>
       <c r="J28">
-        <v>5.45</v>
+        <v>10045</v>
       </c>
       <c r="K28">
-        <v>550</v>
+        <v>5.44</v>
+      </c>
+      <c r="L28">
+        <v>546</v>
       </c>
     </row>
     <row r="29">
@@ -1398,34 +1483,37 @@
         <v>2026-02-28</v>
       </c>
       <c r="B29">
-        <v>20649606</v>
+        <v>54960000</v>
       </c>
       <c r="C29">
-        <v>172</v>
+        <v>458</v>
       </c>
       <c r="D29">
-        <v>2647985</v>
+        <v>144420000</v>
       </c>
       <c r="E29">
-        <v>1122601</v>
+        <v>24540000</v>
       </c>
       <c r="F29">
-        <v>3770586</v>
+        <v>26160000</v>
       </c>
       <c r="G29">
-        <v>447.6</v>
+        <v>195120000</v>
       </c>
       <c r="H29">
-        <v>2</v>
+        <v>-71.8</v>
       </c>
       <c r="I29">
-        <v>7040</v>
+        <v>2</v>
       </c>
       <c r="J29">
-        <v>4.18</v>
+        <v>12935</v>
       </c>
       <c r="K29">
-        <v>294</v>
+        <v>6.64</v>
+      </c>
+      <c r="L29">
+        <v>859</v>
       </c>
     </row>
     <row r="30">
@@ -1433,34 +1521,37 @@
         <v>2026-03-01</v>
       </c>
       <c r="B30">
-        <v>23602362</v>
+        <v>44640000</v>
       </c>
       <c r="C30">
-        <v>197</v>
+        <v>372</v>
       </c>
       <c r="D30">
-        <v>2769921</v>
+        <v>149340000</v>
       </c>
       <c r="E30">
-        <v>1818601</v>
+        <v>16140000</v>
       </c>
       <c r="F30">
-        <v>4588522</v>
+        <v>43800000</v>
       </c>
       <c r="G30">
-        <v>414.4</v>
+        <v>209280000</v>
       </c>
       <c r="H30">
-        <v>2</v>
+        <v>-78.7</v>
       </c>
       <c r="I30">
-        <v>9556</v>
+        <v>2</v>
       </c>
       <c r="J30">
-        <v>5.23</v>
+        <v>9534</v>
       </c>
       <c r="K30">
-        <v>500</v>
+        <v>5.22</v>
+      </c>
+      <c r="L30">
+        <v>498</v>
       </c>
     </row>
     <row r="31">
@@ -1468,34 +1559,37 @@
         <v>2026-03-02</v>
       </c>
       <c r="B31">
-        <v>15334646</v>
+        <v>26640000</v>
       </c>
       <c r="C31">
-        <v>128</v>
+        <v>222</v>
       </c>
       <c r="D31">
-        <v>1038180</v>
+        <v>42420000</v>
       </c>
       <c r="E31">
-        <v>1435890</v>
+        <v>9600000</v>
       </c>
       <c r="F31">
-        <v>2474070</v>
+        <v>24180000</v>
       </c>
       <c r="G31">
-        <v>519.8</v>
+        <v>76200000</v>
       </c>
       <c r="H31">
-        <v>2</v>
+        <v>-65</v>
       </c>
       <c r="I31">
-        <v>6871</v>
+        <v>2</v>
       </c>
       <c r="J31">
-        <v>4.11</v>
+        <v>6887</v>
       </c>
       <c r="K31">
-        <v>282</v>
+        <v>4.12</v>
+      </c>
+      <c r="L31">
+        <v>284</v>
       </c>
     </row>
     <row r="32">
@@ -1503,33 +1597,36 @@
         <v>2026-03-03</v>
       </c>
       <c r="B32">
-        <v>26062992</v>
+        <v>51120000</v>
       </c>
       <c r="C32">
-        <v>217</v>
+        <v>426</v>
       </c>
       <c r="D32">
-        <v>3365094</v>
+        <v>175500000</v>
       </c>
       <c r="E32">
-        <v>1958323</v>
+        <v>16920000</v>
       </c>
       <c r="F32">
-        <v>5323417</v>
+        <v>26100000</v>
       </c>
       <c r="G32">
-        <v>389.6</v>
+        <v>218520000</v>
       </c>
       <c r="H32">
-        <v>2</v>
+        <v>-76.6</v>
       </c>
       <c r="I32">
-        <v>9847</v>
+        <v>2</v>
       </c>
       <c r="J32">
+        <v>9850</v>
+      </c>
+      <c r="K32">
         <v>5.35</v>
       </c>
-      <c r="K32">
+      <c r="L32">
         <v>527</v>
       </c>
     </row>
@@ -1538,34 +1635,37 @@
         <v>2026-03-04</v>
       </c>
       <c r="B33">
-        <v>16712598</v>
+        <v>28320000</v>
       </c>
       <c r="C33">
-        <v>139</v>
+        <v>236</v>
       </c>
       <c r="D33">
-        <v>1438642</v>
+        <v>67740000</v>
       </c>
       <c r="E33">
-        <v>1349862</v>
+        <v>10260000</v>
       </c>
       <c r="F33">
-        <v>2788504</v>
+        <v>22800000</v>
       </c>
       <c r="G33">
-        <v>499.3</v>
+        <v>100800000</v>
       </c>
       <c r="H33">
-        <v>2</v>
+        <v>-71.9</v>
       </c>
       <c r="I33">
-        <v>7210</v>
+        <v>2</v>
       </c>
       <c r="J33">
-        <v>4.25</v>
+        <v>7154</v>
       </c>
       <c r="K33">
-        <v>306</v>
+        <v>4.23</v>
+      </c>
+      <c r="L33">
+        <v>303</v>
       </c>
     </row>
     <row r="34">
@@ -1573,34 +1673,37 @@
         <v>2026-03-05</v>
       </c>
       <c r="B34">
-        <v>14448819</v>
+        <v>23280000</v>
       </c>
       <c r="C34">
-        <v>120</v>
+        <v>194</v>
       </c>
       <c r="D34">
-        <v>2032854</v>
+        <v>58680000</v>
       </c>
       <c r="E34">
-        <v>247101</v>
+        <v>600000</v>
       </c>
       <c r="F34">
-        <v>2279955</v>
+        <v>53700000</v>
       </c>
       <c r="G34">
-        <v>533.7</v>
+        <v>112980000</v>
       </c>
       <c r="H34">
-        <v>0</v>
+        <v>-79.4</v>
       </c>
       <c r="I34">
-        <v>3363</v>
+        <v>1</v>
       </c>
       <c r="J34">
-        <v>2.65</v>
+        <v>3243</v>
       </c>
       <c r="K34">
-        <v>89</v>
+        <v>2.6</v>
+      </c>
+      <c r="L34">
+        <v>84</v>
       </c>
     </row>
     <row r="35">
@@ -1608,34 +1711,37 @@
         <v>2026-03-06</v>
       </c>
       <c r="B35">
-        <v>22125984</v>
+        <v>41760000</v>
       </c>
       <c r="C35">
-        <v>184</v>
+        <v>348</v>
       </c>
       <c r="D35">
-        <v>2863033</v>
+        <v>159240000</v>
       </c>
       <c r="E35">
-        <v>1307802</v>
+        <v>12000000</v>
       </c>
       <c r="F35">
-        <v>4170835</v>
+        <v>5040000</v>
       </c>
       <c r="G35">
-        <v>430.5</v>
+        <v>176280000</v>
       </c>
       <c r="H35">
-        <v>2</v>
+        <v>-76.3</v>
       </c>
       <c r="I35">
-        <v>7839</v>
+        <v>2</v>
       </c>
       <c r="J35">
+        <v>7858</v>
+      </c>
+      <c r="K35">
         <v>4.52</v>
       </c>
-      <c r="K35">
-        <v>354</v>
+      <c r="L35">
+        <v>355</v>
       </c>
     </row>
     <row r="36">
@@ -1643,34 +1749,37 @@
         <v>2026-03-07</v>
       </c>
       <c r="B36">
-        <v>14350394</v>
+        <v>22800000</v>
       </c>
       <c r="C36">
-        <v>120</v>
+        <v>190</v>
       </c>
       <c r="D36">
-        <v>2021685</v>
+        <v>57420000</v>
       </c>
       <c r="E36">
-        <v>237090</v>
+        <v>1020000</v>
       </c>
       <c r="F36">
-        <v>2258775</v>
+        <v>4620000</v>
       </c>
       <c r="G36">
-        <v>535.3</v>
+        <v>63060000</v>
       </c>
       <c r="H36">
-        <v>0</v>
+        <v>-63.8</v>
       </c>
       <c r="I36">
-        <v>3339</v>
+        <v>1</v>
       </c>
       <c r="J36">
-        <v>2.64</v>
+        <v>3413</v>
       </c>
       <c r="K36">
-        <v>88</v>
+        <v>2.67</v>
+      </c>
+      <c r="L36">
+        <v>91</v>
       </c>
     </row>
     <row r="37">
@@ -1678,34 +1787,37 @@
         <v>2026-03-08</v>
       </c>
       <c r="B37">
-        <v>17598425</v>
+        <v>30720000</v>
       </c>
       <c r="C37">
-        <v>147</v>
+        <v>256</v>
       </c>
       <c r="D37">
-        <v>2742045</v>
+        <v>174240000</v>
       </c>
       <c r="E37">
-        <v>256616</v>
+        <v>2640000</v>
       </c>
       <c r="F37">
-        <v>2998661</v>
+        <v>5040000</v>
       </c>
       <c r="G37">
-        <v>486.9</v>
+        <v>181920000</v>
       </c>
       <c r="H37">
-        <v>0</v>
+        <v>-83.1</v>
       </c>
       <c r="I37">
-        <v>3992</v>
+        <v>2</v>
       </c>
       <c r="J37">
-        <v>2.91</v>
+        <v>4069</v>
       </c>
       <c r="K37">
-        <v>116</v>
+        <v>2.95</v>
+      </c>
+      <c r="L37">
+        <v>120</v>
       </c>
     </row>
     <row r="38">
@@ -1713,34 +1825,37 @@
         <v>2026-03-09</v>
       </c>
       <c r="B38">
-        <v>30000000</v>
+        <v>61200000</v>
       </c>
       <c r="C38">
-        <v>250</v>
+        <v>510</v>
       </c>
       <c r="D38">
-        <v>3329290</v>
+        <v>159960000</v>
       </c>
       <c r="E38">
-        <v>3270710</v>
+        <v>26280000</v>
       </c>
       <c r="F38">
-        <v>6600000</v>
+        <v>3000000</v>
       </c>
       <c r="G38">
-        <v>354.5</v>
+        <v>189240000</v>
       </c>
       <c r="H38">
-        <v>2</v>
+        <v>-67.7</v>
       </c>
       <c r="I38">
-        <v>13597</v>
+        <v>2</v>
       </c>
       <c r="J38">
-        <v>6.92</v>
+        <v>13640</v>
       </c>
       <c r="K38">
-        <v>941</v>
+        <v>6.93</v>
+      </c>
+      <c r="L38">
+        <v>945</v>
       </c>
     </row>
     <row r="39">
@@ -1748,34 +1863,37 @@
         <v>2026-03-10</v>
       </c>
       <c r="B39">
-        <v>19468504</v>
+        <v>35520000</v>
       </c>
       <c r="C39">
-        <v>162</v>
+        <v>296</v>
       </c>
       <c r="D39">
-        <v>699041</v>
+        <v>44840000</v>
       </c>
       <c r="E39">
-        <v>2763900</v>
+        <v>29640000</v>
       </c>
       <c r="F39">
-        <v>3462941</v>
+        <v>27540000</v>
       </c>
       <c r="G39">
-        <v>462.2</v>
+        <v>102020000</v>
       </c>
       <c r="H39">
-        <v>2</v>
+        <v>-65.2</v>
       </c>
       <c r="I39">
-        <v>14952</v>
+        <v>2</v>
       </c>
       <c r="J39">
-        <v>7.48</v>
+        <v>15000</v>
       </c>
       <c r="K39">
-        <v>1118</v>
+        <v>7.5</v>
+      </c>
+      <c r="L39">
+        <v>1125</v>
       </c>
     </row>
     <row r="40">
@@ -1783,34 +1901,37 @@
         <v>2026-03-11</v>
       </c>
       <c r="B40">
-        <v>14940945</v>
+        <v>24240000</v>
       </c>
       <c r="C40">
-        <v>125</v>
+        <v>202</v>
       </c>
       <c r="D40">
-        <v>504112</v>
+        <v>25980000</v>
       </c>
       <c r="E40">
-        <v>1882910</v>
+        <v>15900000</v>
       </c>
       <c r="F40">
-        <v>2387022</v>
+        <v>21060000</v>
       </c>
       <c r="G40">
-        <v>525.9</v>
+        <v>62940000</v>
       </c>
       <c r="H40">
-        <v>2</v>
+        <v>-61.5</v>
       </c>
       <c r="I40">
-        <v>9460</v>
+        <v>2</v>
       </c>
       <c r="J40">
-        <v>5.19</v>
+        <v>9437</v>
       </c>
       <c r="K40">
-        <v>491</v>
+        <v>5.18</v>
+      </c>
+      <c r="L40">
+        <v>489</v>
       </c>
     </row>
     <row r="41">
@@ -1818,34 +1939,37 @@
         <v>2026-03-12</v>
       </c>
       <c r="B41">
-        <v>26161417</v>
+        <v>50880000</v>
       </c>
       <c r="C41">
-        <v>218</v>
+        <v>424</v>
       </c>
       <c r="D41">
-        <v>2688137</v>
+        <v>136920000</v>
       </c>
       <c r="E41">
-        <v>2665684</v>
+        <v>22260000</v>
       </c>
       <c r="F41">
-        <v>5353821</v>
+        <v>19800000</v>
       </c>
       <c r="G41">
-        <v>388.6</v>
+        <v>178980000</v>
       </c>
       <c r="H41">
-        <v>2</v>
+        <v>-71.6</v>
       </c>
       <c r="I41">
-        <v>12121</v>
+        <v>2</v>
       </c>
       <c r="J41">
-        <v>6.3</v>
+        <v>12012</v>
       </c>
       <c r="K41">
-        <v>764</v>
+        <v>6.26</v>
+      </c>
+      <c r="L41">
+        <v>752</v>
       </c>
     </row>
     <row r="42">
@@ -1853,34 +1977,37 @@
         <v>2026-03-13</v>
       </c>
       <c r="B42">
-        <v>21338583</v>
+        <v>38400000</v>
       </c>
       <c r="C42">
-        <v>178</v>
+        <v>320</v>
       </c>
       <c r="D42">
-        <v>2373558</v>
+        <v>121440000</v>
       </c>
       <c r="E42">
-        <v>1581641</v>
+        <v>13680000</v>
       </c>
       <c r="F42">
-        <v>3955199</v>
+        <v>18540000</v>
       </c>
       <c r="G42">
-        <v>439.5</v>
+        <v>153660000</v>
       </c>
       <c r="H42">
-        <v>2</v>
+        <v>-75</v>
       </c>
       <c r="I42">
-        <v>8395</v>
+        <v>2</v>
       </c>
       <c r="J42">
-        <v>4.75</v>
+        <v>8538</v>
       </c>
       <c r="K42">
-        <v>399</v>
+        <v>4.81</v>
+      </c>
+      <c r="L42">
+        <v>411</v>
       </c>
     </row>
     <row r="43">
@@ -1888,34 +2015,37 @@
         <v>2026-03-14</v>
       </c>
       <c r="B43">
-        <v>21830709</v>
+        <v>41040000</v>
       </c>
       <c r="C43">
-        <v>182</v>
+        <v>342</v>
       </c>
       <c r="D43">
-        <v>1916686</v>
+        <v>106320000</v>
       </c>
       <c r="E43">
-        <v>2172704</v>
+        <v>19800000</v>
       </c>
       <c r="F43">
-        <v>4089390</v>
+        <v>22800000</v>
       </c>
       <c r="G43">
-        <v>433.8</v>
+        <v>148920000</v>
       </c>
       <c r="H43">
-        <v>2</v>
+        <v>-72.4</v>
       </c>
       <c r="I43">
-        <v>11081</v>
+        <v>2</v>
       </c>
       <c r="J43">
-        <v>5.87</v>
+        <v>11016</v>
       </c>
       <c r="K43">
-        <v>650</v>
+        <v>5.84</v>
+      </c>
+      <c r="L43">
+        <v>643</v>
       </c>
     </row>
     <row r="44">
@@ -1923,33 +2053,36 @@
         <v>2026-03-15</v>
       </c>
       <c r="B44">
-        <v>25374016</v>
+        <v>49680000</v>
       </c>
       <c r="C44">
-        <v>211</v>
+        <v>414</v>
       </c>
       <c r="D44">
-        <v>3259719</v>
+        <v>176160000</v>
       </c>
       <c r="E44">
-        <v>1853045</v>
+        <v>16560000</v>
       </c>
       <c r="F44">
-        <v>5112764</v>
+        <v>780000</v>
       </c>
       <c r="G44">
-        <v>396.3</v>
+        <v>193500000</v>
       </c>
       <c r="H44">
-        <v>2</v>
+        <v>-74.3</v>
       </c>
       <c r="I44">
-        <v>9702</v>
+        <v>2</v>
       </c>
       <c r="J44">
+        <v>9704</v>
+      </c>
+      <c r="K44">
         <v>5.29</v>
       </c>
-      <c r="K44">
+      <c r="L44">
         <v>513</v>
       </c>
     </row>
@@ -1958,34 +2091,37 @@
         <v>2026-03-16</v>
       </c>
       <c r="B45">
-        <v>17696850</v>
+        <v>58080000</v>
       </c>
       <c r="C45">
-        <v>147</v>
+        <v>484</v>
       </c>
       <c r="D45">
-        <v>2409222</v>
+        <v>123960000</v>
       </c>
       <c r="E45">
-        <v>613177</v>
+        <v>27180000</v>
       </c>
       <c r="F45">
-        <v>3022399</v>
+        <v>15720000</v>
       </c>
       <c r="G45">
-        <v>485.5</v>
+        <v>166860000</v>
       </c>
       <c r="H45">
-        <v>1</v>
+        <v>-65.2</v>
       </c>
       <c r="I45">
-        <v>5032</v>
+        <v>2</v>
       </c>
       <c r="J45">
-        <v>3.35</v>
+        <v>14004</v>
       </c>
       <c r="K45">
-        <v>169</v>
+        <v>7.09</v>
+      </c>
+      <c r="L45">
+        <v>993</v>
       </c>
     </row>
     <row r="46">
@@ -1993,34 +2129,37 @@
         <v>2026-03-17</v>
       </c>
       <c r="B46">
-        <v>13366142</v>
+        <v>20400000</v>
       </c>
       <c r="C46">
-        <v>111</v>
+        <v>170</v>
       </c>
       <c r="D46">
-        <v>285773</v>
+        <v>15060000</v>
       </c>
       <c r="E46">
-        <v>1765456</v>
+        <v>15000000</v>
       </c>
       <c r="F46">
-        <v>2051229</v>
+        <v>26100000</v>
       </c>
       <c r="G46">
-        <v>551.6</v>
+        <v>56160000</v>
       </c>
       <c r="H46">
-        <v>2</v>
+        <v>-63.7</v>
       </c>
       <c r="I46">
-        <v>9218</v>
+        <v>2</v>
       </c>
       <c r="J46">
-        <v>5.09</v>
+        <v>9073</v>
       </c>
       <c r="K46">
-        <v>469</v>
+        <v>5.03</v>
+      </c>
+      <c r="L46">
+        <v>456</v>
       </c>
     </row>
     <row r="47">
@@ -2028,34 +2167,37 @@
         <v>2026-03-18</v>
       </c>
       <c r="B47">
-        <v>19665354</v>
+        <v>35520000</v>
       </c>
       <c r="C47">
-        <v>164</v>
+        <v>296</v>
       </c>
       <c r="D47">
-        <v>1976738</v>
+        <v>105660000</v>
       </c>
       <c r="E47">
-        <v>1536702</v>
+        <v>11160000</v>
       </c>
       <c r="F47">
-        <v>3513440</v>
+        <v>27600000</v>
       </c>
       <c r="G47">
-        <v>459.7</v>
+        <v>144420000</v>
       </c>
       <c r="H47">
-        <v>2</v>
+        <v>-75.4</v>
       </c>
       <c r="I47">
-        <v>8444</v>
+        <v>2</v>
       </c>
       <c r="J47">
-        <v>4.77</v>
+        <v>7518</v>
       </c>
       <c r="K47">
-        <v>403</v>
+        <v>4.38</v>
+      </c>
+      <c r="L47">
+        <v>329</v>
       </c>
     </row>
     <row r="48">
@@ -2063,34 +2205,37 @@
         <v>2026-03-19</v>
       </c>
       <c r="B48">
-        <v>15433071</v>
+        <v>25440000</v>
       </c>
       <c r="C48">
-        <v>129</v>
+        <v>212</v>
       </c>
       <c r="D48">
-        <v>1480409</v>
+        <v>53700000</v>
       </c>
       <c r="E48">
-        <v>1015617</v>
+        <v>24420000</v>
       </c>
       <c r="F48">
-        <v>2496026</v>
+        <v>37620000</v>
       </c>
       <c r="G48">
-        <v>518.3</v>
+        <v>115740000</v>
       </c>
       <c r="H48">
-        <v>2</v>
+        <v>-78</v>
       </c>
       <c r="I48">
-        <v>5395</v>
+        <v>2</v>
       </c>
       <c r="J48">
-        <v>3.5</v>
+        <v>12887</v>
       </c>
       <c r="K48">
-        <v>189</v>
+        <v>6.62</v>
+      </c>
+      <c r="L48">
+        <v>853</v>
       </c>
     </row>
     <row r="49">
@@ -2098,34 +2243,37 @@
         <v>2026-03-20</v>
       </c>
       <c r="B49">
-        <v>27834646</v>
+        <v>55920000</v>
       </c>
       <c r="C49">
-        <v>232</v>
+        <v>466</v>
       </c>
       <c r="D49">
-        <v>2888948</v>
+        <v>143940000</v>
       </c>
       <c r="E49">
-        <v>2993587</v>
+        <v>24720000</v>
       </c>
       <c r="F49">
-        <v>5882535</v>
+        <v>11340000</v>
       </c>
       <c r="G49">
-        <v>373.2</v>
+        <v>180000000</v>
       </c>
       <c r="H49">
-        <v>2</v>
+        <v>-68.9</v>
       </c>
       <c r="I49">
-        <v>13040</v>
+        <v>2</v>
       </c>
       <c r="J49">
-        <v>6.68</v>
+        <v>13008</v>
       </c>
       <c r="K49">
-        <v>871</v>
+        <v>6.67</v>
+      </c>
+      <c r="L49">
+        <v>868</v>
       </c>
     </row>
     <row r="50">
@@ -2133,34 +2281,37 @@
         <v>2026-03-21</v>
       </c>
       <c r="B50">
-        <v>19566929</v>
+        <v>34320000</v>
       </c>
       <c r="C50">
-        <v>163</v>
+        <v>286</v>
       </c>
       <c r="D50">
-        <v>2448569</v>
+        <v>136620000</v>
       </c>
       <c r="E50">
-        <v>1039583</v>
+        <v>6300000</v>
       </c>
       <c r="F50">
-        <v>3488152</v>
+        <v>29580000</v>
       </c>
       <c r="G50">
-        <v>461</v>
+        <v>172500000</v>
       </c>
       <c r="H50">
-        <v>2</v>
+        <v>-80.1</v>
       </c>
       <c r="I50">
-        <v>6823</v>
+        <v>2</v>
       </c>
       <c r="J50">
-        <v>4.09</v>
+        <v>5551</v>
       </c>
       <c r="K50">
-        <v>279</v>
+        <v>3.56</v>
+      </c>
+      <c r="L50">
+        <v>198</v>
       </c>
     </row>
     <row r="51">
@@ -2168,34 +2319,37 @@
         <v>2026-03-22</v>
       </c>
       <c r="B51">
-        <v>14547244</v>
+        <v>23040000</v>
       </c>
       <c r="C51">
-        <v>121</v>
+        <v>192</v>
       </c>
       <c r="D51">
-        <v>1106827</v>
+        <v>39720000</v>
       </c>
       <c r="E51">
-        <v>1194387</v>
+        <v>7440000</v>
       </c>
       <c r="F51">
-        <v>2301214</v>
+        <v>14520000</v>
       </c>
       <c r="G51">
-        <v>532.2</v>
+        <v>61680000</v>
       </c>
       <c r="H51">
-        <v>2</v>
+        <v>-62.6</v>
       </c>
       <c r="I51">
-        <v>5831</v>
+        <v>2</v>
       </c>
       <c r="J51">
-        <v>3.68</v>
+        <v>6012</v>
       </c>
       <c r="K51">
-        <v>215</v>
+        <v>3.76</v>
+      </c>
+      <c r="L51">
+        <v>226</v>
       </c>
     </row>
     <row r="52">
@@ -2203,34 +2357,37 @@
         <v>2026-03-23</v>
       </c>
       <c r="B52">
-        <v>16220472</v>
+        <v>27120000</v>
       </c>
       <c r="C52">
-        <v>135</v>
+        <v>226</v>
       </c>
       <c r="D52">
-        <v>2416967</v>
+        <v>119520000</v>
       </c>
       <c r="E52">
-        <v>257495</v>
+        <v>2340000</v>
       </c>
       <c r="F52">
-        <v>2674462</v>
+        <v>20580000</v>
       </c>
       <c r="G52">
-        <v>506.5</v>
+        <v>142440000</v>
       </c>
       <c r="H52">
-        <v>0</v>
+        <v>-81</v>
       </c>
       <c r="I52">
-        <v>3750</v>
+        <v>2</v>
       </c>
       <c r="J52">
-        <v>2.81</v>
+        <v>3947</v>
       </c>
       <c r="K52">
-        <v>105</v>
+        <v>2.89</v>
+      </c>
+      <c r="L52">
+        <v>114</v>
       </c>
     </row>
     <row r="53">
@@ -2238,33 +2395,36 @@
         <v>2026-03-24</v>
       </c>
       <c r="B53">
-        <v>15531496</v>
+        <v>24240000</v>
       </c>
       <c r="C53">
-        <v>129</v>
+        <v>202</v>
       </c>
       <c r="D53">
-        <v>1578486</v>
+        <v>60240000</v>
       </c>
       <c r="E53">
-        <v>939573</v>
+        <v>5760000</v>
       </c>
       <c r="F53">
-        <v>2518059</v>
+        <v>1980000</v>
       </c>
       <c r="G53">
-        <v>516.8</v>
+        <v>67980000</v>
       </c>
       <c r="H53">
-        <v>2</v>
+        <v>-64.3</v>
       </c>
       <c r="I53">
-        <v>5323</v>
+        <v>2</v>
       </c>
       <c r="J53">
+        <v>5332</v>
+      </c>
+      <c r="K53">
         <v>3.47</v>
       </c>
-      <c r="K53">
+      <c r="L53">
         <v>185</v>
       </c>
     </row>
@@ -2273,34 +2433,37 @@
         <v>2026-03-25</v>
       </c>
       <c r="B54">
-        <v>27244094</v>
+        <v>52800000</v>
       </c>
       <c r="C54">
-        <v>227</v>
+        <v>440</v>
       </c>
       <c r="D54">
-        <v>2642893</v>
+        <v>129900000</v>
       </c>
       <c r="E54">
-        <v>3050479</v>
+        <v>24540000</v>
       </c>
       <c r="F54">
-        <v>5693372</v>
+        <v>23640000</v>
       </c>
       <c r="G54">
-        <v>378.5</v>
+        <v>178080000</v>
       </c>
       <c r="H54">
-        <v>2</v>
+        <v>-70.4</v>
       </c>
       <c r="I54">
-        <v>13089</v>
+        <v>2</v>
       </c>
       <c r="J54">
-        <v>6.7</v>
+        <v>12935</v>
       </c>
       <c r="K54">
-        <v>877</v>
+        <v>6.64</v>
+      </c>
+      <c r="L54">
+        <v>859</v>
       </c>
     </row>
     <row r="55">
@@ -2308,33 +2471,36 @@
         <v>2026-03-26</v>
       </c>
       <c r="B55">
-        <v>25866142</v>
+        <v>53280000</v>
       </c>
       <c r="C55">
-        <v>216</v>
+        <v>444</v>
       </c>
       <c r="D55">
-        <v>2093625</v>
+        <v>109860000</v>
       </c>
       <c r="E55">
-        <v>3169218</v>
+        <v>27600000</v>
       </c>
       <c r="F55">
-        <v>5262843</v>
+        <v>34620000</v>
       </c>
       <c r="G55">
-        <v>391.5</v>
+        <v>172080000</v>
       </c>
       <c r="H55">
-        <v>2</v>
+        <v>-69</v>
       </c>
       <c r="I55">
-        <v>14177</v>
+        <v>2</v>
       </c>
       <c r="J55">
+        <v>14174</v>
+      </c>
+      <c r="K55">
         <v>7.16</v>
       </c>
-      <c r="K55">
+      <c r="L55">
         <v>1015</v>
       </c>
     </row>
@@ -2343,34 +2509,37 @@
         <v>2026-03-27</v>
       </c>
       <c r="B56">
-        <v>24881890</v>
+        <v>48480000</v>
       </c>
       <c r="C56">
-        <v>207</v>
+        <v>404</v>
       </c>
       <c r="D56">
-        <v>2990521</v>
+        <v>157680000</v>
       </c>
       <c r="E56">
-        <v>1974102</v>
+        <v>17040000</v>
       </c>
       <c r="F56">
-        <v>4964623</v>
+        <v>9360000</v>
       </c>
       <c r="G56">
-        <v>401.2</v>
+        <v>184080000</v>
       </c>
       <c r="H56">
-        <v>2</v>
+        <v>-73.7</v>
       </c>
       <c r="I56">
-        <v>9968</v>
+        <v>2</v>
       </c>
       <c r="J56">
-        <v>5.4</v>
+        <v>9899</v>
       </c>
       <c r="K56">
-        <v>538</v>
+        <v>5.37</v>
+      </c>
+      <c r="L56">
+        <v>532</v>
       </c>
     </row>
     <row r="57">
@@ -2378,34 +2547,37 @@
         <v>2026-03-28</v>
       </c>
       <c r="B57">
-        <v>28326772</v>
+        <v>56160000</v>
       </c>
       <c r="C57">
-        <v>236</v>
+        <v>468</v>
       </c>
       <c r="D57">
-        <v>2431580</v>
+        <v>119160000</v>
       </c>
       <c r="E57">
-        <v>3610721</v>
+        <v>29640000</v>
       </c>
       <c r="F57">
-        <v>6042301</v>
+        <v>36240000</v>
       </c>
       <c r="G57">
-        <v>368.8</v>
+        <v>185040000</v>
       </c>
       <c r="H57">
-        <v>2</v>
+        <v>-69.6</v>
       </c>
       <c r="I57">
-        <v>14952</v>
+        <v>2</v>
       </c>
       <c r="J57">
-        <v>7.48</v>
+        <v>15000</v>
       </c>
       <c r="K57">
-        <v>1118</v>
+        <v>7.5</v>
+      </c>
+      <c r="L57">
+        <v>1125</v>
       </c>
     </row>
     <row r="58">
@@ -2413,34 +2585,37 @@
         <v>2026-03-29</v>
       </c>
       <c r="B58">
-        <v>10413386</v>
+        <v>13440000</v>
       </c>
       <c r="C58">
-        <v>87</v>
+        <v>112</v>
       </c>
       <c r="D58">
-        <v>60985</v>
+        <v>4440000</v>
       </c>
       <c r="E58">
-        <v>1414108</v>
+        <v>16920000</v>
       </c>
       <c r="F58">
-        <v>1475093</v>
+        <v>24720000</v>
       </c>
       <c r="G58">
-        <v>605.9</v>
+        <v>46080000</v>
       </c>
       <c r="H58">
-        <v>2</v>
+        <v>-70.8</v>
       </c>
       <c r="I58">
-        <v>9798</v>
+        <v>2</v>
       </c>
       <c r="J58">
-        <v>5.33</v>
+        <v>9850</v>
       </c>
       <c r="K58">
-        <v>522</v>
+        <v>5.35</v>
+      </c>
+      <c r="L58">
+        <v>527</v>
       </c>
     </row>
     <row r="59">
@@ -2448,34 +2623,37 @@
         <v>2026-03-30</v>
       </c>
       <c r="B59">
-        <v>17992126</v>
+        <v>32400000</v>
       </c>
       <c r="C59">
-        <v>150</v>
+        <v>270</v>
       </c>
       <c r="D59">
-        <v>1667066</v>
+        <v>82080000</v>
       </c>
       <c r="E59">
-        <v>1427013</v>
+        <v>11520000</v>
       </c>
       <c r="F59">
-        <v>3094079</v>
+        <v>9540000</v>
       </c>
       <c r="G59">
-        <v>481.5</v>
+        <v>103140000</v>
       </c>
       <c r="H59">
-        <v>2</v>
+        <v>-68.6</v>
       </c>
       <c r="I59">
-        <v>7645</v>
+        <v>2</v>
       </c>
       <c r="J59">
+        <v>7664</v>
+      </c>
+      <c r="K59">
         <v>4.44</v>
       </c>
-      <c r="K59">
-        <v>339</v>
+      <c r="L59">
+        <v>340</v>
       </c>
     </row>
     <row r="60">
@@ -2483,34 +2661,37 @@
         <v>2026-03-31</v>
       </c>
       <c r="B60">
-        <v>28425197</v>
+        <v>56400000</v>
       </c>
       <c r="C60">
-        <v>237</v>
+        <v>470</v>
       </c>
       <c r="D60">
-        <v>2523972</v>
+        <v>126480000</v>
       </c>
       <c r="E60">
-        <v>3550515</v>
+        <v>29580000</v>
       </c>
       <c r="F60">
-        <v>6074487</v>
+        <v>22440000</v>
       </c>
       <c r="G60">
-        <v>367.9</v>
+        <v>178500000</v>
       </c>
       <c r="H60">
-        <v>2</v>
+        <v>-68.4</v>
       </c>
       <c r="I60">
-        <v>15000</v>
+        <v>2</v>
       </c>
       <c r="J60">
-        <v>7.5</v>
+        <v>14976</v>
       </c>
       <c r="K60">
-        <v>1125</v>
+        <v>7.49</v>
+      </c>
+      <c r="L60">
+        <v>1122</v>
       </c>
     </row>
     <row r="61">
@@ -2518,34 +2699,37 @@
         <v>2026-04-01</v>
       </c>
       <c r="B61">
-        <v>23110236</v>
+        <v>43200000</v>
       </c>
       <c r="C61">
-        <v>193</v>
+        <v>360</v>
       </c>
       <c r="D61">
-        <v>2413499</v>
+        <v>126420000</v>
       </c>
       <c r="E61">
-        <v>2033857</v>
+        <v>10260000</v>
       </c>
       <c r="F61">
-        <v>4447356</v>
+        <v>13260000</v>
       </c>
       <c r="G61">
-        <v>419.6</v>
+        <v>149940000</v>
       </c>
       <c r="H61">
-        <v>2</v>
+        <v>-71.2</v>
       </c>
       <c r="I61">
-        <v>10137</v>
+        <v>2</v>
       </c>
       <c r="J61">
-        <v>5.47</v>
+        <v>7154</v>
       </c>
       <c r="K61">
-        <v>554</v>
+        <v>4.23</v>
+      </c>
+      <c r="L61">
+        <v>303</v>
       </c>
     </row>
     <row r="62">
@@ -2553,33 +2737,36 @@
         <v>2026-04-02</v>
       </c>
       <c r="B62">
-        <v>12972441</v>
+        <v>19440000</v>
       </c>
       <c r="C62">
-        <v>108</v>
+        <v>162</v>
       </c>
       <c r="D62">
-        <v>1543989</v>
+        <v>32040000</v>
       </c>
       <c r="E62">
-        <v>426392</v>
+        <v>1200000</v>
       </c>
       <c r="F62">
-        <v>1970381</v>
+        <v>12720000</v>
       </c>
       <c r="G62">
-        <v>558.4</v>
+        <v>45960000</v>
       </c>
       <c r="H62">
-        <v>1</v>
+        <v>-57.7</v>
       </c>
       <c r="I62">
-        <v>3484</v>
+        <v>2</v>
       </c>
       <c r="J62">
+        <v>3486</v>
+      </c>
+      <c r="K62">
         <v>2.7</v>
       </c>
-      <c r="K62">
+      <c r="L62">
         <v>94</v>
       </c>
     </row>
@@ -2588,34 +2775,37 @@
         <v>2026-04-03</v>
       </c>
       <c r="B63">
-        <v>28818898</v>
+        <v>58320000</v>
       </c>
       <c r="C63">
-        <v>240</v>
+        <v>486</v>
       </c>
       <c r="D63">
-        <v>3135648</v>
+        <v>156900000</v>
       </c>
       <c r="E63">
-        <v>3068357</v>
+        <v>25440000</v>
       </c>
       <c r="F63">
-        <v>6204005</v>
+        <v>32520000</v>
       </c>
       <c r="G63">
-        <v>364.5</v>
+        <v>214860000</v>
       </c>
       <c r="H63">
-        <v>2</v>
+        <v>-72.9</v>
       </c>
       <c r="I63">
-        <v>13331</v>
+        <v>2</v>
       </c>
       <c r="J63">
-        <v>6.8</v>
+        <v>13300</v>
       </c>
       <c r="K63">
-        <v>907</v>
+        <v>6.79</v>
+      </c>
+      <c r="L63">
+        <v>903</v>
       </c>
     </row>
     <row r="64">
@@ -2623,34 +2813,37 @@
         <v>2026-04-04</v>
       </c>
       <c r="B64">
-        <v>20452756</v>
+        <v>36000000</v>
       </c>
       <c r="C64">
-        <v>170</v>
+        <v>300</v>
       </c>
       <c r="D64">
-        <v>2664321</v>
+        <v>143940000</v>
       </c>
       <c r="E64">
-        <v>1054216</v>
+        <v>9180000</v>
       </c>
       <c r="F64">
-        <v>3718537</v>
+        <v>16260000</v>
       </c>
       <c r="G64">
-        <v>450</v>
+        <v>169380000</v>
       </c>
       <c r="H64">
-        <v>2</v>
+        <v>-78.7</v>
       </c>
       <c r="I64">
-        <v>6750</v>
+        <v>2</v>
       </c>
       <c r="J64">
-        <v>4.06</v>
+        <v>6717</v>
       </c>
       <c r="K64">
-        <v>274</v>
+        <v>4.05</v>
+      </c>
+      <c r="L64">
+        <v>272</v>
       </c>
     </row>
     <row r="65">
@@ -2658,34 +2851,37 @@
         <v>2026-04-05</v>
       </c>
       <c r="B65">
-        <v>18779528</v>
+        <v>33600000</v>
       </c>
       <c r="C65">
-        <v>156</v>
+        <v>280</v>
       </c>
       <c r="D65">
-        <v>1202578</v>
+        <v>61800000</v>
       </c>
       <c r="E65">
-        <v>2086057</v>
+        <v>17520000</v>
       </c>
       <c r="F65">
-        <v>3288635</v>
+        <v>10440000</v>
       </c>
       <c r="G65">
-        <v>471</v>
+        <v>89760000</v>
       </c>
       <c r="H65">
-        <v>2</v>
+        <v>-62.6</v>
       </c>
       <c r="I65">
-        <v>10161</v>
+        <v>2</v>
       </c>
       <c r="J65">
-        <v>5.48</v>
+        <v>10093</v>
       </c>
       <c r="K65">
-        <v>557</v>
+        <v>5.46</v>
+      </c>
+      <c r="L65">
+        <v>551</v>
       </c>
     </row>
     <row r="66">
@@ -2693,34 +2889,37 @@
         <v>2026-04-06</v>
       </c>
       <c r="B66">
-        <v>22716535</v>
+        <v>43200000</v>
       </c>
       <c r="C66">
-        <v>189</v>
+        <v>360</v>
       </c>
       <c r="D66">
-        <v>1467343</v>
+        <v>78540000</v>
       </c>
       <c r="E66">
-        <v>2868474</v>
+        <v>25200000</v>
       </c>
       <c r="F66">
-        <v>4335817</v>
+        <v>17460000</v>
       </c>
       <c r="G66">
-        <v>423.9</v>
+        <v>121200000</v>
       </c>
       <c r="H66">
-        <v>2</v>
+        <v>-64.4</v>
       </c>
       <c r="I66">
-        <v>13355</v>
+        <v>2</v>
       </c>
       <c r="J66">
-        <v>6.81</v>
+        <v>13202</v>
       </c>
       <c r="K66">
-        <v>909</v>
+        <v>6.75</v>
+      </c>
+      <c r="L66">
+        <v>891</v>
       </c>
     </row>
     <row r="67">
@@ -2728,34 +2927,37 @@
         <v>2026-04-07</v>
       </c>
       <c r="B67">
-        <v>14153543</v>
+        <v>22320000</v>
       </c>
       <c r="C67">
-        <v>118</v>
+        <v>186</v>
       </c>
       <c r="D67">
-        <v>1204452</v>
+        <v>41520000</v>
       </c>
       <c r="E67">
-        <v>1012193</v>
+        <v>5640000</v>
       </c>
       <c r="F67">
-        <v>2216645</v>
+        <v>480000</v>
       </c>
       <c r="G67">
-        <v>538.5</v>
+        <v>47640000</v>
       </c>
       <c r="H67">
-        <v>2</v>
+        <v>-53.1</v>
       </c>
       <c r="I67">
-        <v>5250</v>
+        <v>2</v>
       </c>
       <c r="J67">
-        <v>3.44</v>
+        <v>5283</v>
       </c>
       <c r="K67">
-        <v>181</v>
+        <v>3.45</v>
+      </c>
+      <c r="L67">
+        <v>182</v>
       </c>
     </row>
     <row r="68">
@@ -2763,34 +2965,37 @@
         <v>2026-04-08</v>
       </c>
       <c r="B68">
-        <v>14350394</v>
+        <v>23040000</v>
       </c>
       <c r="C68">
-        <v>120</v>
+        <v>192</v>
       </c>
       <c r="D68">
-        <v>395171</v>
+        <v>18660000</v>
       </c>
       <c r="E68">
-        <v>1863604</v>
+        <v>14640000</v>
       </c>
       <c r="F68">
-        <v>2258775</v>
+        <v>23700000</v>
       </c>
       <c r="G68">
-        <v>535.3</v>
+        <v>57000000</v>
       </c>
       <c r="H68">
-        <v>2</v>
+        <v>-59.6</v>
       </c>
       <c r="I68">
-        <v>8952</v>
+        <v>2</v>
       </c>
       <c r="J68">
-        <v>4.98</v>
+        <v>8927</v>
       </c>
       <c r="K68">
-        <v>446</v>
+        <v>4.97</v>
+      </c>
+      <c r="L68">
+        <v>444</v>
       </c>
     </row>
     <row r="69">
@@ -2798,34 +3003,37 @@
         <v>2026-04-09</v>
       </c>
       <c r="B69">
-        <v>18188976</v>
+        <v>32880000</v>
       </c>
       <c r="C69">
-        <v>152</v>
+        <v>274</v>
       </c>
       <c r="D69">
-        <v>1919245</v>
+        <v>83700000</v>
       </c>
       <c r="E69">
-        <v>1223008</v>
+        <v>8940000</v>
       </c>
       <c r="F69">
-        <v>3142253</v>
+        <v>6420000</v>
       </c>
       <c r="G69">
-        <v>478.9</v>
+        <v>99060000</v>
       </c>
       <c r="H69">
-        <v>2</v>
+        <v>-66.8</v>
       </c>
       <c r="I69">
-        <v>6508</v>
+        <v>2</v>
       </c>
       <c r="J69">
-        <v>3.96</v>
+        <v>6619</v>
       </c>
       <c r="K69">
-        <v>258</v>
+        <v>4.01</v>
+      </c>
+      <c r="L69">
+        <v>265</v>
       </c>
     </row>
     <row r="70">
@@ -2833,34 +3041,37 @@
         <v>2026-04-10</v>
       </c>
       <c r="B70">
-        <v>23602362</v>
+        <v>44160000</v>
       </c>
       <c r="C70">
-        <v>197</v>
+        <v>368</v>
       </c>
       <c r="D70">
-        <v>2702222</v>
+        <v>142680000</v>
       </c>
       <c r="E70">
-        <v>1886300</v>
+        <v>16920000</v>
       </c>
       <c r="F70">
-        <v>4588522</v>
+        <v>6840000</v>
       </c>
       <c r="G70">
-        <v>414.4</v>
+        <v>166440000</v>
       </c>
       <c r="H70">
-        <v>2</v>
+        <v>-73.5</v>
       </c>
       <c r="I70">
-        <v>9653</v>
+        <v>2</v>
       </c>
       <c r="J70">
-        <v>5.27</v>
+        <v>9850</v>
       </c>
       <c r="K70">
-        <v>509</v>
+        <v>5.35</v>
+      </c>
+      <c r="L70">
+        <v>527</v>
       </c>
     </row>
     <row r="71">
@@ -2868,34 +3079,37 @@
         <v>2026-04-11</v>
       </c>
       <c r="B71">
-        <v>26948819</v>
+        <v>53520000</v>
       </c>
       <c r="C71">
-        <v>225</v>
+        <v>446</v>
       </c>
       <c r="D71">
-        <v>2531392</v>
+        <v>130200000</v>
       </c>
       <c r="E71">
-        <v>3068445</v>
+        <v>25740000</v>
       </c>
       <c r="F71">
-        <v>5599837</v>
+        <v>29520000</v>
       </c>
       <c r="G71">
-        <v>381.2</v>
+        <v>185460000</v>
       </c>
       <c r="H71">
-        <v>2</v>
+        <v>-71.1</v>
       </c>
       <c r="I71">
-        <v>13621</v>
+        <v>2</v>
       </c>
       <c r="J71">
-        <v>6.93</v>
+        <v>13421</v>
       </c>
       <c r="K71">
-        <v>944</v>
+        <v>6.84</v>
+      </c>
+      <c r="L71">
+        <v>918</v>
       </c>
     </row>
     <row r="72">
@@ -2903,34 +3117,37 @@
         <v>2026-04-12</v>
       </c>
       <c r="B72">
-        <v>23011811</v>
+        <v>44640000</v>
       </c>
       <c r="C72">
-        <v>192</v>
+        <v>372</v>
       </c>
       <c r="D72">
-        <v>2296363</v>
+        <v>119520000</v>
       </c>
       <c r="E72">
-        <v>2122992</v>
+        <v>18360000</v>
       </c>
       <c r="F72">
-        <v>4419355</v>
+        <v>22740000</v>
       </c>
       <c r="G72">
-        <v>420.7</v>
+        <v>160620000</v>
       </c>
       <c r="H72">
-        <v>2</v>
+        <v>-72.2</v>
       </c>
       <c r="I72">
-        <v>10403</v>
+        <v>2</v>
       </c>
       <c r="J72">
-        <v>5.58</v>
+        <v>10433</v>
       </c>
       <c r="K72">
-        <v>580</v>
+        <v>5.6</v>
+      </c>
+      <c r="L72">
+        <v>584</v>
       </c>
     </row>
     <row r="73">
@@ -2938,34 +3155,37 @@
         <v>2026-04-13</v>
       </c>
       <c r="B73">
-        <v>17204724</v>
+        <v>29760000</v>
       </c>
       <c r="C73">
-        <v>143</v>
+        <v>248</v>
       </c>
       <c r="D73">
-        <v>1615704</v>
+        <v>65700000</v>
       </c>
       <c r="E73">
-        <v>1288779</v>
+        <v>8640000</v>
       </c>
       <c r="F73">
-        <v>2904483</v>
+        <v>19380000</v>
       </c>
       <c r="G73">
-        <v>492.4</v>
+        <v>93720000</v>
       </c>
       <c r="H73">
-        <v>2</v>
+        <v>-68.2</v>
       </c>
       <c r="I73">
-        <v>6460</v>
+        <v>2</v>
       </c>
       <c r="J73">
-        <v>3.94</v>
+        <v>6498</v>
       </c>
       <c r="K73">
-        <v>255</v>
+        <v>3.96</v>
+      </c>
+      <c r="L73">
+        <v>257</v>
       </c>
     </row>
     <row r="74">
@@ -2973,34 +3193,37 @@
         <v>2026-04-14</v>
       </c>
       <c r="B74">
-        <v>13661417</v>
+        <v>19440000</v>
       </c>
       <c r="C74">
-        <v>114</v>
+        <v>162</v>
       </c>
       <c r="D74">
-        <v>251560</v>
+        <v>16080000</v>
       </c>
       <c r="E74">
-        <v>1861119</v>
+        <v>2520000</v>
       </c>
       <c r="F74">
-        <v>2112679</v>
+        <v>34800000</v>
       </c>
       <c r="G74">
-        <v>546.6</v>
+        <v>53400000</v>
       </c>
       <c r="H74">
-        <v>2</v>
+        <v>-63.6</v>
       </c>
       <c r="I74">
-        <v>10984</v>
+        <v>2</v>
       </c>
       <c r="J74">
-        <v>5.83</v>
+        <v>4020</v>
       </c>
       <c r="K74">
-        <v>640</v>
+        <v>2.93</v>
+      </c>
+      <c r="L74">
+        <v>118</v>
       </c>
     </row>
     <row r="75">
@@ -3008,34 +3231,37 @@
         <v>2026-04-15</v>
       </c>
       <c r="B75">
-        <v>15826772</v>
+        <v>26400000</v>
       </c>
       <c r="C75">
-        <v>132</v>
+        <v>220</v>
       </c>
       <c r="D75">
-        <v>2013835</v>
+        <v>77760000</v>
       </c>
       <c r="E75">
-        <v>570789</v>
+        <v>3720000</v>
       </c>
       <c r="F75">
-        <v>2584624</v>
+        <v>19380000</v>
       </c>
       <c r="G75">
-        <v>512.3</v>
+        <v>100860000</v>
       </c>
       <c r="H75">
-        <v>1</v>
+        <v>-73.8</v>
       </c>
       <c r="I75">
-        <v>4379</v>
+        <v>2</v>
       </c>
       <c r="J75">
-        <v>3.07</v>
+        <v>4506</v>
       </c>
       <c r="K75">
-        <v>134</v>
+        <v>3.13</v>
+      </c>
+      <c r="L75">
+        <v>141</v>
       </c>
     </row>
     <row r="76">
@@ -3043,34 +3269,37 @@
         <v>2026-04-16</v>
       </c>
       <c r="B76">
-        <v>21732283</v>
+        <v>40800000</v>
       </c>
       <c r="C76">
-        <v>181</v>
+        <v>340</v>
       </c>
       <c r="D76">
-        <v>2395111</v>
+        <v>128040000</v>
       </c>
       <c r="E76">
-        <v>1667286</v>
+        <v>14400000</v>
       </c>
       <c r="F76">
-        <v>4062397</v>
+        <v>34200000</v>
       </c>
       <c r="G76">
+        <v>176640000</v>
+      </c>
+      <c r="H76">
+        <v>-76.9</v>
+      </c>
+      <c r="I76">
+        <v>2</v>
+      </c>
+      <c r="J76">
+        <v>8830</v>
+      </c>
+      <c r="K76">
+        <v>4.93</v>
+      </c>
+      <c r="L76">
         <v>435</v>
-      </c>
-      <c r="H76">
-        <v>2</v>
-      </c>
-      <c r="I76">
-        <v>8952</v>
-      </c>
-      <c r="J76">
-        <v>4.98</v>
-      </c>
-      <c r="K76">
-        <v>446</v>
       </c>
     </row>
     <row r="77">
@@ -3078,34 +3307,37 @@
         <v>2026-04-17</v>
       </c>
       <c r="B77">
-        <v>13562992</v>
+        <v>20880000</v>
       </c>
       <c r="C77">
-        <v>113</v>
+        <v>174</v>
       </c>
       <c r="D77">
-        <v>126949</v>
+        <v>10200000</v>
       </c>
       <c r="E77">
-        <v>1965169</v>
+        <v>22860000</v>
       </c>
       <c r="F77">
-        <v>2092118</v>
+        <v>39840000</v>
       </c>
       <c r="G77">
-        <v>548.3</v>
+        <v>72900000</v>
       </c>
       <c r="H77">
-        <v>2</v>
+        <v>-71.4</v>
       </c>
       <c r="I77">
-        <v>13573</v>
+        <v>2</v>
       </c>
       <c r="J77">
-        <v>6.91</v>
+        <v>12255</v>
       </c>
       <c r="K77">
-        <v>938</v>
+        <v>6.36</v>
+      </c>
+      <c r="L77">
+        <v>779</v>
       </c>
     </row>
     <row r="78">
@@ -3113,34 +3345,37 @@
         <v>2026-04-18</v>
       </c>
       <c r="B78">
-        <v>11791339</v>
+        <v>16320000</v>
       </c>
       <c r="C78">
-        <v>98</v>
+        <v>136</v>
       </c>
       <c r="D78">
-        <v>1195784</v>
+        <v>16620000</v>
       </c>
       <c r="E78">
-        <v>539493</v>
+        <v>840000</v>
       </c>
       <c r="F78">
-        <v>1735277</v>
+        <v>12420000</v>
       </c>
       <c r="G78">
-        <v>579.5</v>
+        <v>29880000</v>
       </c>
       <c r="H78">
-        <v>1</v>
+        <v>-45.4</v>
       </c>
       <c r="I78">
-        <v>3387</v>
+        <v>2</v>
       </c>
       <c r="J78">
-        <v>2.66</v>
+        <v>3340</v>
       </c>
       <c r="K78">
-        <v>90</v>
+        <v>2.64</v>
+      </c>
+      <c r="L78">
+        <v>88</v>
       </c>
     </row>
     <row r="79">
@@ -3148,34 +3383,37 @@
         <v>2026-04-19</v>
       </c>
       <c r="B79">
-        <v>18976378</v>
+        <v>33600000</v>
       </c>
       <c r="C79">
-        <v>158</v>
+        <v>280</v>
       </c>
       <c r="D79">
-        <v>1376868</v>
+        <v>72300000</v>
       </c>
       <c r="E79">
-        <v>1961181</v>
+        <v>17280000</v>
       </c>
       <c r="F79">
-        <v>3338049</v>
+        <v>8460000</v>
       </c>
       <c r="G79">
-        <v>468.5</v>
+        <v>98040000</v>
       </c>
       <c r="H79">
-        <v>2</v>
+        <v>-65.7</v>
       </c>
       <c r="I79">
-        <v>9895</v>
+        <v>2</v>
       </c>
       <c r="J79">
-        <v>5.37</v>
+        <v>9996</v>
       </c>
       <c r="K79">
-        <v>531</v>
+        <v>5.41</v>
+      </c>
+      <c r="L79">
+        <v>541</v>
       </c>
     </row>
     <row r="80">
@@ -3183,34 +3421,37 @@
         <v>2026-04-20</v>
       </c>
       <c r="B80">
-        <v>10216535</v>
+        <v>12720000</v>
       </c>
       <c r="C80">
-        <v>85</v>
+        <v>106</v>
       </c>
       <c r="D80">
-        <v>41934</v>
+        <v>3240000</v>
       </c>
       <c r="E80">
-        <v>1397230</v>
+        <v>17640000</v>
       </c>
       <c r="F80">
-        <v>1439164</v>
+        <v>5280000</v>
       </c>
       <c r="G80">
-        <v>609.9</v>
+        <v>26160000</v>
       </c>
       <c r="H80">
-        <v>2</v>
+        <v>-51.4</v>
       </c>
       <c r="I80">
-        <v>10234</v>
+        <v>2</v>
       </c>
       <c r="J80">
-        <v>5.51</v>
+        <v>10142</v>
       </c>
       <c r="K80">
-        <v>564</v>
+        <v>5.48</v>
+      </c>
+      <c r="L80">
+        <v>556</v>
       </c>
     </row>
     <row r="81">
@@ -3218,34 +3459,37 @@
         <v>2026-04-21</v>
       </c>
       <c r="B81">
-        <v>15826772</v>
+        <v>27360000</v>
       </c>
       <c r="C81">
-        <v>132</v>
+        <v>228</v>
       </c>
       <c r="D81">
-        <v>1822425</v>
+        <v>69720000</v>
       </c>
       <c r="E81">
-        <v>762199</v>
+        <v>8640000</v>
       </c>
       <c r="F81">
-        <v>2584624</v>
+        <v>5520000</v>
       </c>
       <c r="G81">
-        <v>512.3</v>
+        <v>83880000</v>
       </c>
       <c r="H81">
-        <v>1</v>
+        <v>-67.4</v>
       </c>
       <c r="I81">
-        <v>4863</v>
+        <v>2</v>
       </c>
       <c r="J81">
-        <v>3.28</v>
+        <v>6498</v>
       </c>
       <c r="K81">
-        <v>160</v>
+        <v>3.96</v>
+      </c>
+      <c r="L81">
+        <v>257</v>
       </c>
     </row>
     <row r="82">
@@ -3253,34 +3497,37 @@
         <v>2026-04-22</v>
       </c>
       <c r="B82">
-        <v>16614173</v>
+        <v>28320000</v>
       </c>
       <c r="C82">
-        <v>138</v>
+        <v>236</v>
       </c>
       <c r="D82">
-        <v>890070</v>
+        <v>45780000</v>
       </c>
       <c r="E82">
-        <v>1875470</v>
+        <v>16260000</v>
       </c>
       <c r="F82">
-        <v>2765540</v>
+        <v>13380000</v>
       </c>
       <c r="G82">
-        <v>500.8</v>
+        <v>75420000</v>
       </c>
       <c r="H82">
-        <v>2</v>
+        <v>-62.5</v>
       </c>
       <c r="I82">
-        <v>9460</v>
+        <v>2</v>
       </c>
       <c r="J82">
-        <v>5.19</v>
+        <v>9583</v>
       </c>
       <c r="K82">
-        <v>491</v>
+        <v>5.24</v>
+      </c>
+      <c r="L82">
+        <v>502</v>
       </c>
     </row>
     <row r="83">
@@ -3288,34 +3535,37 @@
         <v>2026-04-23</v>
       </c>
       <c r="B83">
-        <v>17106299</v>
+        <v>41280000</v>
       </c>
       <c r="C83">
-        <v>143</v>
+        <v>344</v>
       </c>
       <c r="D83">
-        <v>2587572</v>
+        <v>143640000</v>
       </c>
       <c r="E83">
-        <v>293560</v>
+        <v>21600000</v>
       </c>
       <c r="F83">
-        <v>2881132</v>
+        <v>30000000</v>
       </c>
       <c r="G83">
-        <v>493.7</v>
+        <v>195240000</v>
       </c>
       <c r="H83">
-        <v>0</v>
+        <v>-78.9</v>
       </c>
       <c r="I83">
-        <v>3992</v>
+        <v>2</v>
       </c>
       <c r="J83">
-        <v>2.91</v>
+        <v>11745</v>
       </c>
       <c r="K83">
-        <v>116</v>
+        <v>6.14</v>
+      </c>
+      <c r="L83">
+        <v>721</v>
       </c>
     </row>
     <row r="84">
@@ -3323,34 +3573,37 @@
         <v>2026-04-24</v>
       </c>
       <c r="B84">
-        <v>16122047</v>
+        <v>26640000</v>
       </c>
       <c r="C84">
-        <v>134</v>
+        <v>222</v>
       </c>
       <c r="D84">
-        <v>1006493</v>
+        <v>45000000</v>
       </c>
       <c r="E84">
-        <v>1645393</v>
+        <v>6240000</v>
       </c>
       <c r="F84">
-        <v>2651886</v>
+        <v>16980000</v>
       </c>
       <c r="G84">
-        <v>507.9</v>
+        <v>68220000</v>
       </c>
       <c r="H84">
-        <v>2</v>
+        <v>-60.9</v>
       </c>
       <c r="I84">
-        <v>7911</v>
+        <v>2</v>
       </c>
       <c r="J84">
-        <v>4.55</v>
+        <v>5526</v>
       </c>
       <c r="K84">
-        <v>360</v>
+        <v>3.55</v>
+      </c>
+      <c r="L84">
+        <v>196</v>
       </c>
     </row>
     <row r="85">
@@ -3358,34 +3611,37 @@
         <v>2026-04-25</v>
       </c>
       <c r="B85">
-        <v>18385827</v>
+        <v>30480000</v>
       </c>
       <c r="C85">
-        <v>153</v>
+        <v>254</v>
       </c>
       <c r="D85">
-        <v>651974</v>
+        <v>40860000</v>
       </c>
       <c r="E85">
-        <v>2538763</v>
+        <v>26280000</v>
       </c>
       <c r="F85">
-        <v>3190737</v>
+        <v>21840000</v>
       </c>
       <c r="G85">
-        <v>476.2</v>
+        <v>88980000</v>
       </c>
       <c r="H85">
-        <v>2</v>
+        <v>-65.7</v>
       </c>
       <c r="I85">
-        <v>13766</v>
+        <v>2</v>
       </c>
       <c r="J85">
-        <v>6.99</v>
+        <v>13640</v>
       </c>
       <c r="K85">
-        <v>962</v>
+        <v>6.93</v>
+      </c>
+      <c r="L85">
+        <v>945</v>
       </c>
     </row>
     <row r="86">
@@ -3393,34 +3649,37 @@
         <v>2026-04-26</v>
       </c>
       <c r="B86">
-        <v>26358268</v>
+        <v>50880000</v>
       </c>
       <c r="C86">
-        <v>220</v>
+        <v>424</v>
       </c>
       <c r="D86">
-        <v>2454672</v>
+        <v>128040000</v>
       </c>
       <c r="E86">
-        <v>2960188</v>
+        <v>19860000</v>
       </c>
       <c r="F86">
-        <v>5414860</v>
+        <v>54000000</v>
       </c>
       <c r="G86">
-        <v>386.8</v>
+        <v>201900000</v>
       </c>
       <c r="H86">
-        <v>2</v>
+        <v>-74.8</v>
       </c>
       <c r="I86">
-        <v>13403</v>
+        <v>2</v>
       </c>
       <c r="J86">
-        <v>6.83</v>
+        <v>11040</v>
       </c>
       <c r="K86">
-        <v>915</v>
+        <v>5.85</v>
+      </c>
+      <c r="L86">
+        <v>646</v>
       </c>
     </row>
     <row r="87">
@@ -3428,34 +3687,37 @@
         <v>2026-04-27</v>
       </c>
       <c r="B87">
-        <v>19960630</v>
+        <v>51840000</v>
       </c>
       <c r="C87">
-        <v>166</v>
+        <v>432</v>
       </c>
       <c r="D87">
-        <v>2273525</v>
+        <v>115800000</v>
       </c>
       <c r="E87">
-        <v>1316245</v>
+        <v>21000000</v>
       </c>
       <c r="F87">
-        <v>3589770</v>
+        <v>37740000</v>
       </c>
       <c r="G87">
-        <v>456</v>
+        <v>174540000</v>
       </c>
       <c r="H87">
-        <v>2</v>
+        <v>-70.3</v>
       </c>
       <c r="I87">
-        <v>7452</v>
+        <v>2</v>
       </c>
       <c r="J87">
-        <v>4.35</v>
+        <v>11502</v>
       </c>
       <c r="K87">
-        <v>324</v>
+        <v>6.04</v>
+      </c>
+      <c r="L87">
+        <v>695</v>
       </c>
     </row>
     <row r="88">
@@ -3463,34 +3725,37 @@
         <v>2026-04-28</v>
       </c>
       <c r="B88">
-        <v>16811024</v>
+        <v>22560000</v>
       </c>
       <c r="C88">
-        <v>140</v>
+        <v>188</v>
       </c>
       <c r="D88">
-        <v>886383</v>
+        <v>45780000</v>
       </c>
       <c r="E88">
-        <v>1925161</v>
+        <v>1380000</v>
       </c>
       <c r="F88">
-        <v>2811544</v>
+        <v>5580000</v>
       </c>
       <c r="G88">
-        <v>497.9</v>
+        <v>52740000</v>
       </c>
       <c r="H88">
-        <v>2</v>
+        <v>-57.2</v>
       </c>
       <c r="I88">
-        <v>9653</v>
+        <v>2</v>
       </c>
       <c r="J88">
-        <v>5.27</v>
+        <v>3559</v>
       </c>
       <c r="K88">
-        <v>509</v>
+        <v>2.73</v>
+      </c>
+      <c r="L88">
+        <v>97</v>
       </c>
     </row>
     <row r="89">
@@ -3498,34 +3763,37 @@
         <v>2026-04-29</v>
       </c>
       <c r="B89">
-        <v>20748031</v>
+        <v>27840000</v>
       </c>
       <c r="C89">
-        <v>173</v>
+        <v>232</v>
       </c>
       <c r="D89">
-        <v>1187409</v>
+        <v>66180000</v>
       </c>
       <c r="E89">
-        <v>2609317</v>
+        <v>3360000</v>
       </c>
       <c r="F89">
-        <v>3796726</v>
+        <v>15000000</v>
       </c>
       <c r="G89">
-        <v>446.5</v>
+        <v>84540000</v>
       </c>
       <c r="H89">
-        <v>2</v>
+        <v>-67.1</v>
       </c>
       <c r="I89">
-        <v>12823</v>
+        <v>2</v>
       </c>
       <c r="J89">
-        <v>6.59</v>
+        <v>4360</v>
       </c>
       <c r="K89">
-        <v>845</v>
+        <v>3.07</v>
+      </c>
+      <c r="L89">
+        <v>134</v>
       </c>
     </row>
     <row r="90">
@@ -3533,34 +3801,37 @@
         <v>2026-04-30</v>
       </c>
       <c r="B90">
-        <v>17696850</v>
+        <v>29280000</v>
       </c>
       <c r="C90">
-        <v>147</v>
+        <v>244</v>
       </c>
       <c r="D90">
-        <v>1101983</v>
+        <v>52680000</v>
       </c>
       <c r="E90">
-        <v>1920416</v>
+        <v>3240000</v>
       </c>
       <c r="F90">
-        <v>3022399</v>
+        <v>44280000</v>
       </c>
       <c r="G90">
-        <v>485.5</v>
+        <v>100200000</v>
       </c>
       <c r="H90">
-        <v>2</v>
+        <v>-70.8</v>
       </c>
       <c r="I90">
-        <v>9169</v>
+        <v>2</v>
       </c>
       <c r="J90">
-        <v>5.07</v>
+        <v>4312</v>
       </c>
       <c r="K90">
-        <v>465</v>
+        <v>3.05</v>
+      </c>
+      <c r="L90">
+        <v>132</v>
       </c>
     </row>
     <row r="91">
@@ -3568,39 +3839,42 @@
         <v>2026-05-01</v>
       </c>
       <c r="B91">
-        <v>21437008</v>
+        <v>40080000</v>
       </c>
       <c r="C91">
-        <v>179</v>
+        <v>334</v>
       </c>
       <c r="D91">
-        <v>1104957</v>
+        <v>65820000</v>
       </c>
       <c r="E91">
-        <v>2876925</v>
+        <v>17760000</v>
       </c>
       <c r="F91">
-        <v>3981882</v>
+        <v>22980000</v>
       </c>
       <c r="G91">
-        <v>438.4</v>
+        <v>106560000</v>
       </c>
       <c r="H91">
-        <v>2</v>
+        <v>-62.4</v>
       </c>
       <c r="I91">
-        <v>14565</v>
+        <v>2</v>
       </c>
       <c r="J91">
-        <v>7.32</v>
+        <v>10190</v>
       </c>
       <c r="K91">
-        <v>1066</v>
+        <v>5.5</v>
+      </c>
+      <c r="L91">
+        <v>560</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K91"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L91"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3652,7 +3926,7 @@
         <v>Số quan sát</v>
       </c>
       <c r="B6" t="str">
-        <v>200 observations (dùng 90 ngày đầu)</v>
+        <v>197 observations (dùng 90 ngày đầu)</v>
       </c>
     </row>
     <row r="7">

</xml_diff>